<commit_message>
Add Operations Staff as third SUS evaluation role (3+3+3 distribution)
Redistribute 9 participants equally across all 3 platform stakeholder
groups per Chinese Smart Park OSS model:
  P1-P3: IPDC Management Staff
  P4-P6: Tenant Representative
  P7-P9: Operations Staff

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/research/SUS_Evaluation_IPDC_OSS.xlsx
+++ b/data/research/SUS_Evaluation_IPDC_OSS.xlsx
@@ -1469,12 +1469,12 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t>IPDC Management Staff</t>
+          <t>Tenant Representative</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>Adama SEZ</t>
+          <t>Hawassa SEZ</t>
         </is>
       </c>
       <c r="E6" s="26" t="inlineStr">
@@ -1504,12 +1504,12 @@
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Hawassa SEZ</t>
+          <t>Adama SEZ</t>
         </is>
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>Smartphone (Chrome)</t>
+          <t>Smartphone (Opera)</t>
         </is>
       </c>
       <c r="F7" s="25" t="inlineStr">
@@ -1534,12 +1534,12 @@
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>Adama SEZ</t>
+          <t>Bole Lemi SEZ</t>
         </is>
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>Smartphone (Opera)</t>
+          <t>Laptop (Chrome)</t>
         </is>
       </c>
       <c r="F8" s="26" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
-          <t>Laptop (Chrome)</t>
+          <t>Smartphone (Chrome)</t>
         </is>
       </c>
       <c r="F9" s="25" t="inlineStr">
@@ -1589,17 +1589,17 @@
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>Kombolcha SEZ</t>
+          <t>Hawassa SEZ</t>
         </is>
       </c>
       <c r="E10" s="26" t="inlineStr">
         <is>
-          <t>Smartphone (Chrome)</t>
+          <t>Smartphone (Opera)</t>
         </is>
       </c>
       <c r="F10" s="26" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D11" s="25" t="inlineStr">
         <is>
-          <t>Hawassa SEZ</t>
+          <t>Adama SEZ</t>
         </is>
       </c>
       <c r="E11" s="25" t="inlineStr">
         <is>
-          <t>Smartphone (Opera)</t>
+          <t>Smartphone (Chrome)</t>
         </is>
       </c>
       <c r="F11" s="25" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>IPDC Management Staff</t>
+          <t>Tenant Representative</t>
         </is>
       </c>
       <c r="D8" s="35" t="n"/>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D11" s="35" t="n"/>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D12" s="35" t="n"/>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D13" s="35" t="n"/>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>IPDC Management Staff</t>
+          <t>Tenant Representative</t>
         </is>
       </c>
       <c r="D7" s="45">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D10" s="35">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="C11" s="26" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D11" s="45">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D12" s="35">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t>IPDC Management Staff</t>
+          <t>Tenant Representative</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Smartphone (Chrome)</t>
+          <t>Smartphone (Opera)</t>
         </is>
       </c>
       <c r="E7" s="49">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>Smartphone (Opera)</t>
+          <t>Laptop (Chrome)</t>
         </is>
       </c>
       <c r="E8" s="49">
@@ -3110,12 +3110,12 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>Laptop (Chrome)</t>
+          <t>Smartphone (Chrome)</t>
         </is>
       </c>
       <c r="E9" s="49">
@@ -3142,12 +3142,12 @@
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>Smartphone (Chrome)</t>
+          <t>Smartphone (Opera)</t>
         </is>
       </c>
       <c r="E10" s="49">
@@ -3174,12 +3174,12 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D11" s="25" t="inlineStr">
         <is>
-          <t>Smartphone (Opera)</t>
+          <t>Smartphone (Chrome)</t>
         </is>
       </c>
       <c r="E11" s="49">

</xml_diff>

<commit_message>
Update SUS evaluation workbook and generator for 9-section Google Form
- generate_sus_excel.py: updated task scenarios to role-differentiated sets
  (M1-M4 Management, T1-T4 Tenant, O1-O4 Operations, X1-X4 Offline/all roles);
  expanded Participant Profiles with Investment Type and Sector columns for
  tenant participants (P4-P6); added Sheet 6 Offline Experience with Q8b
  (6 role-labelled offline task columns, Section 6 of 9) and Q19/Q20
  (Section 8 of 9) with MEAN(Q19) auto-calculation; corrected all section
  and question number references throughout to match final 9-section form
- SUS_Evaluation_IPDC_OSS.xlsx: regenerated from updated script

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/research/SUS_Evaluation_IPDC_OSS.xlsx
+++ b/data/research/SUS_Evaluation_IPDC_OSS.xlsx
@@ -12,6 +12,7 @@
     <sheet name="SUS Raw Responses" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="SUS Score Calculation" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Summary &amp; Results" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Offline Experience" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -286,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -437,6 +438,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -945,7 +961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -997,7 +1013,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>This sheet — purpose, SUS formula, scoring guide, task scenarios</t>
+          <t>This sheet — purpose, SUS formula, scoring guide, role-differentiated task scenarios</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1025,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Participant IDs, roles, industrial parks, devices used (10-Feb-2026)</t>
+          <t>P1–P9 roles, parks, devices, and tenant company profile (investment type, sector)</t>
         </is>
       </c>
     </row>
@@ -1049,264 +1065,494 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Offline Experience</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Supplementary Q8b/Q19/Q20 responses — offline tasks attempted, confidence score, clarity</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>SUS SCORING FORMULA</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Odd items — Positive (Q1,Q3,Q5,Q7,Q9):</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Converted score  =  Raw response  −  1</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Even items — Negative (Q2,Q4,Q6,Q8,Q10):</t>
+          <t>Odd items — Positive (Q1,Q3,Q5,Q7,Q9):</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Converted score  =  5  −  Raw response</t>
+          <t>Converted score  =  Raw response  −  1</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>SUS Score:</t>
+          <t>Even items — Negative (Q2,Q4,Q6,Q8,Q10):</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Sum of all 10 converted scores  ×  2.5</t>
+          <t>Converted score  =  5  −  Raw response</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="7" t="inlineStr">
         <is>
+          <t>SUS Score:</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Sum of all 10 converted scores  ×  2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
           <t>Scale:</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>0 (worst)  →  100 (best)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>SUS SCORE INTERPRETATION (Bangor et al. / Sauro)</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="B21" s="9" t="inlineStr">
+    <row r="22" ht="16" customHeight="1">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>&gt; 85.5</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Excellent</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="B22" s="11" t="inlineStr">
+    <row r="23" ht="16" customHeight="1">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>72.6 – 85.5</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="B23" s="13" t="inlineStr">
+    <row r="24" ht="16" customHeight="1">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>52.0 – 72.5</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="B24" s="15" t="inlineStr">
+    <row r="25" ht="16" customHeight="1">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>51.7 – 51.9</t>
         </is>
       </c>
-      <c r="C24" s="16" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>Poor</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="B25" s="17" t="inlineStr">
+    <row r="26" ht="16" customHeight="1">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>&lt; 51.6</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>Awful</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>TASK SCENARIOS ADMINISTERED TO PARTICIPANTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>Task 1</t>
-        </is>
-      </c>
-      <c r="C28" s="20" t="inlineStr">
-        <is>
-          <t>Sign in and navigate the dashboard</t>
-        </is>
-      </c>
-      <c r="D28" s="21" t="inlineStr">
-        <is>
-          <t>Log in using provided credentials and locate the service request list.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>Task 2</t>
+          <t>Task M1</t>
         </is>
       </c>
       <c r="C29" s="20" t="inlineStr">
         <is>
-          <t>Submit a service request</t>
+          <t>[Management] Review and process a service request</t>
         </is>
       </c>
       <c r="D29" s="21" t="inlineStr">
         <is>
-          <t>Create a new maintenance request, set a priority level, add a description, and submit.</t>
+          <t>Log in as Admin, open a pending service request, review the details, and approve or reject it with a stated reason.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Task 3</t>
+          <t>Task M2</t>
         </is>
       </c>
       <c r="C30" s="20" t="inlineStr">
         <is>
-          <t>Check token balance</t>
+          <t>[Management] Resolve a tenant complaint</t>
         </is>
       </c>
       <c r="D30" s="21" t="inlineStr">
         <is>
-          <t>Locate the token dashboard and review the current balance and transaction history.</t>
+          <t>Navigate to Complaint Management, open a pending complaint, select a resolution action, add resolution notes, and confirm.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>Task 4</t>
+          <t>Task M3</t>
         </is>
       </c>
       <c r="C31" s="20" t="inlineStr">
         <is>
-          <t>View an announcement</t>
+          <t>[Management] Publish a park-wide announcement</t>
         </is>
       </c>
       <c r="D31" s="21" t="inlineStr">
         <is>
-          <t>Find the announcements section and read the most recent park notice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="22" t="inlineStr">
+          <t>Create a new announcement with a title, body text, and priority level, then publish it to all park users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>Task M4</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>[Management] View request analytics dashboard</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>Navigate to the admin dashboard and review the summary statistics, request counts by status, and charts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t>Task T1</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>[Tenant] Submit a new service request</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>Log in as Tenant, select a service category, fill in the request details and priority, attach a document if available, and submit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>Task T2</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="inlineStr">
+        <is>
+          <t>[Tenant] Check token balance and transaction history</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>Locate the token section on the dashboard and review the current balance and the list of past transactions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>Task T3</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="inlineStr">
+        <is>
+          <t>[Tenant] File a complaint on a completed service</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>Navigate to My Complaints, select a completed request, choose a complaint category and severity, describe the issue, and submit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>Task T4</t>
+        </is>
+      </c>
+      <c r="C36" s="20" t="inlineStr">
+        <is>
+          <t>[Tenant] Read an in-app bell notification</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>Click the notification bell icon, open an unread notification, and confirm the message content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>Task O1</t>
+        </is>
+      </c>
+      <c r="C37" s="20" t="inlineStr">
+        <is>
+          <t>[Operations] Accept a task from the approved queue</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr">
+        <is>
+          <t>Log in as Operations Staff, open the Approved Requests tab, select a request, and mark it as In Progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="B38" s="19" t="inlineStr">
+        <is>
+          <t>Task O2</t>
+        </is>
+      </c>
+      <c r="C38" s="20" t="inlineStr">
+        <is>
+          <t>[Operations] Complete a task and confirm token deduction</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="inlineStr">
+        <is>
+          <t>Mark an in-progress task as completed, confirm the token amount to deduct from the tenant, and submit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="B39" s="19" t="inlineStr">
+        <is>
+          <t>Task O3</t>
+        </is>
+      </c>
+      <c r="C39" s="20" t="inlineStr">
+        <is>
+          <t>[Operations] Review completed task history</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>Navigate to the Completed tab and review the list of previously fulfilled tasks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>Task O4</t>
+        </is>
+      </c>
+      <c r="C40" s="20" t="inlineStr">
+        <is>
+          <t>[Operations] Read a park announcement</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>Open the Announcements tab in the Operations dashboard and read the latest park-wide notice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="19" t="inlineStr">
+        <is>
+          <t>Task X1</t>
+        </is>
+      </c>
+      <c r="C41" s="20" t="inlineStr">
+        <is>
+          <t>[All Roles] Browse dashboard while offline</t>
+        </is>
+      </c>
+      <c r="D41" s="21" t="inlineStr">
+        <is>
+          <t>Facilitator enables airplane mode. Participant navigates the dashboard and confirms data is still visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="B42" s="19" t="inlineStr">
+        <is>
+          <t>Task X2</t>
+        </is>
+      </c>
+      <c r="C42" s="20" t="inlineStr">
+        <is>
+          <t>[All Roles] Submit a request or action while offline</t>
+        </is>
+      </c>
+      <c r="D42" s="21" t="inlineStr">
+        <is>
+          <t>While offline, perform a key action (submit request / complete task). Confirm the item queues locally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="B43" s="19" t="inlineStr">
+        <is>
+          <t>Task X3</t>
+        </is>
+      </c>
+      <c r="C43" s="20" t="inlineStr">
+        <is>
+          <t>[All Roles] Offline re-login with cached credentials</t>
+        </is>
+      </c>
+      <c r="D43" s="21" t="inlineStr">
+        <is>
+          <t>While offline, log out then log back in using the same credentials. Confirm the system authenticates from cache.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="B44" s="19" t="inlineStr">
+        <is>
+          <t>Task X4</t>
+        </is>
+      </c>
+      <c r="C44" s="20" t="inlineStr">
+        <is>
+          <t>[All Roles] Sync confirmation on reconnection</t>
+        </is>
+      </c>
+      <c r="D44" s="21" t="inlineStr">
+        <is>
+          <t>Facilitator restores network. Participant confirms the sync banner appears and queued items are uploaded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="36" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
         <is>
           <t>⚠  IMPORTANT: Enter REAL participant responses in the 'SUS Raw Responses' sheet. All SUS scores in the thesis must reflect actual collected data. Scores in 'SUS Score Calculation' and 'Summary &amp; Results' update automatically.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="41">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="B9"/>
-    <mergeCell ref="C15:D15"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A20:D20"/>
     <mergeCell ref="D30"/>
+    <mergeCell ref="D39"/>
+    <mergeCell ref="D33"/>
+    <mergeCell ref="D42"/>
+    <mergeCell ref="D38"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="C18:D18"/>
     <mergeCell ref="D29"/>
+    <mergeCell ref="D35"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C16:D16"/>
+    <mergeCell ref="D44"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="D34"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="D31"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="C12:D12"/>
+    <mergeCell ref="D40"/>
     <mergeCell ref="B12"/>
+    <mergeCell ref="D36"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="B11"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="C17:D17"/>
+    <mergeCell ref="A46:D46"/>
     <mergeCell ref="C8:D8"/>
+    <mergeCell ref="D41"/>
     <mergeCell ref="B8"/>
-    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="D32"/>
+    <mergeCell ref="B13"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="D43"/>
     <mergeCell ref="B10"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="D28"/>
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="D37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1318,15 +1564,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1364,7 +1612,17 @@
       </c>
       <c r="F2" s="24" t="inlineStr">
         <is>
-          <t>Date of Evaluation</t>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="G2" s="24" t="inlineStr">
+        <is>
+          <t>Investment Type *</t>
+        </is>
+      </c>
+      <c r="H2" s="24" t="inlineStr">
+        <is>
+          <t>Industry Sector *</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1652,17 @@
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>10 February 2026</t>
+          <t>10 Feb 2026</t>
+        </is>
+      </c>
+      <c r="G3" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1692,17 @@
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>10 February 2026</t>
+          <t>10 Feb 2026</t>
+        </is>
+      </c>
+      <c r="G4" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1732,17 @@
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>10 February 2026</t>
+          <t>10 Feb 2026</t>
+        </is>
+      </c>
+      <c r="G5" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1772,17 @@
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>10 February 2026</t>
+          <t>10 Feb 2026</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>Foreign-invested</t>
+        </is>
+      </c>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>Garment &amp; Textile</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1812,17 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>10 February 2026</t>
+          <t>10 Feb 2026</t>
+        </is>
+      </c>
+      <c r="G7" s="25" t="inlineStr">
+        <is>
+          <t>Local (Ethiopian)</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="inlineStr">
+        <is>
+          <t>Agro-processing &amp; Food</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1852,17 @@
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>10 February 2026</t>
+          <t>10 Feb 2026</t>
+        </is>
+      </c>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>Joint Venture</t>
+        </is>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>Light Manufacturing</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1892,17 @@
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>10 February 2026</t>
+          <t>10 Feb 2026</t>
+        </is>
+      </c>
+      <c r="G9" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1932,17 @@
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>10 February 2026</t>
+          <t>10 Feb 2026</t>
+        </is>
+      </c>
+      <c r="G10" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1634,21 +1972,31 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>10 February 2026</t>
+          <t>10 Feb 2026</t>
+        </is>
+      </c>
+      <c r="G11" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>Note: Participant IDs (P1–P9) are pseudonymised to protect privacy. Signed consent forms are held by the researcher and available on request.</t>
+          <t>Note: Participant IDs (P1–P9) are pseudonymised. * Investment Type and Sector apply to Tenant Representatives (P4–P6) only. Signed consent forms are held by the researcher and available on request.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3230,4 +3578,501 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Offline Experience — Supplementary Data (Q8b, Q19, Q20 from Google Form)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="52" t="inlineStr">
+        <is>
+          <t>These questions are supplementary to the SUS — they do NOT affect the SUS score calculation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="53" t="inlineStr">
+        <is>
+          <t>Q8b — Offline Tasks Attempted (tick = attempted)  |  Google Form: Section 6 of 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="37" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="37" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
+          <t>Browsed dashboard offline (All)</t>
+        </is>
+      </c>
+      <c r="E4" s="37" t="inlineStr">
+        <is>
+          <t>Submitted request offline (Tenant)</t>
+        </is>
+      </c>
+      <c r="F4" s="37" t="inlineStr">
+        <is>
+          <t>Completed task offline (Operations)</t>
+        </is>
+      </c>
+      <c r="G4" s="37" t="inlineStr">
+        <is>
+          <t>Reviewed request offline (Management)</t>
+        </is>
+      </c>
+      <c r="H4" s="37" t="inlineStr">
+        <is>
+          <t>Offline re-login (All)</t>
+        </is>
+      </c>
+      <c r="I4" s="37" t="inlineStr">
+        <is>
+          <t>Sync banner on reconnect (All)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>IPDC Management Staff</t>
+        </is>
+      </c>
+      <c r="D5" s="54" t="n"/>
+      <c r="E5" s="54" t="n"/>
+      <c r="F5" s="54" t="n"/>
+      <c r="G5" s="54" t="n"/>
+      <c r="H5" s="54" t="n"/>
+      <c r="I5" s="54" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>IPDC Management Staff</t>
+        </is>
+      </c>
+      <c r="D6" s="54" t="n"/>
+      <c r="E6" s="54" t="n"/>
+      <c r="F6" s="54" t="n"/>
+      <c r="G6" s="54" t="n"/>
+      <c r="H6" s="54" t="n"/>
+      <c r="I6" s="54" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>IPDC Management Staff</t>
+        </is>
+      </c>
+      <c r="D7" s="54" t="n"/>
+      <c r="E7" s="54" t="n"/>
+      <c r="F7" s="54" t="n"/>
+      <c r="G7" s="54" t="n"/>
+      <c r="H7" s="54" t="n"/>
+      <c r="I7" s="54" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Tenant Representative</t>
+        </is>
+      </c>
+      <c r="D8" s="54" t="n"/>
+      <c r="E8" s="54" t="n"/>
+      <c r="F8" s="54" t="n"/>
+      <c r="G8" s="54" t="n"/>
+      <c r="H8" s="54" t="n"/>
+      <c r="I8" s="54" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>Tenant Representative</t>
+        </is>
+      </c>
+      <c r="D9" s="54" t="n"/>
+      <c r="E9" s="54" t="n"/>
+      <c r="F9" s="54" t="n"/>
+      <c r="G9" s="54" t="n"/>
+      <c r="H9" s="54" t="n"/>
+      <c r="I9" s="54" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Tenant Representative</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="n"/>
+      <c r="E10" s="54" t="n"/>
+      <c r="F10" s="54" t="n"/>
+      <c r="G10" s="54" t="n"/>
+      <c r="H10" s="54" t="n"/>
+      <c r="I10" s="54" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>Operations Staff</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="n"/>
+      <c r="E11" s="54" t="n"/>
+      <c r="F11" s="54" t="n"/>
+      <c r="G11" s="54" t="n"/>
+      <c r="H11" s="54" t="n"/>
+      <c r="I11" s="54" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Operations Staff</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="n"/>
+      <c r="E12" s="54" t="n"/>
+      <c r="F12" s="54" t="n"/>
+      <c r="G12" s="54" t="n"/>
+      <c r="H12" s="54" t="n"/>
+      <c r="I12" s="54" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>Operations Staff</t>
+        </is>
+      </c>
+      <c r="D13" s="54" t="n"/>
+      <c r="E13" s="54" t="n"/>
+      <c r="F13" s="54" t="n"/>
+      <c r="G13" s="54" t="n"/>
+      <c r="H13" s="54" t="n"/>
+      <c r="I13" s="54" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>Enter  ✓  if the participant attempted the task, or leave blank if not attempted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="53" t="inlineStr">
+        <is>
+          <t>Q19 — Offline Confidence Score  |  Q20 — Online/Offline Clarity  |  Google Form: Section 8 of 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="37" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D18" s="37" t="inlineStr">
+        <is>
+          <t>Q19: Offline data confidence (1–5)
+1=Not confident  5=Fully confident</t>
+        </is>
+      </c>
+      <c r="E18" s="37" t="inlineStr">
+        <is>
+          <t>Q20: Online/offline clarity
+Yes always / Sometimes / No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="inlineStr">
+        <is>
+          <t>IPDC Management Staff</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="n"/>
+      <c r="E19" s="35" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>IPDC Management Staff</t>
+        </is>
+      </c>
+      <c r="D20" s="35" t="n"/>
+      <c r="E20" s="35" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" s="25" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>IPDC Management Staff</t>
+        </is>
+      </c>
+      <c r="D21" s="35" t="n"/>
+      <c r="E21" s="35" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Tenant Representative</t>
+        </is>
+      </c>
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="35" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="25" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="inlineStr">
+        <is>
+          <t>Tenant Representative</t>
+        </is>
+      </c>
+      <c r="D23" s="35" t="n"/>
+      <c r="E23" s="35" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Tenant Representative</t>
+        </is>
+      </c>
+      <c r="D24" s="35" t="n"/>
+      <c r="E24" s="35" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="25" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="inlineStr">
+        <is>
+          <t>Operations Staff</t>
+        </is>
+      </c>
+      <c r="D25" s="35" t="n"/>
+      <c r="E25" s="35" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Operations Staff</t>
+        </is>
+      </c>
+      <c r="D26" s="35" t="n"/>
+      <c r="E26" s="35" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" s="25" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="inlineStr">
+        <is>
+          <t>Operations Staff</t>
+        </is>
+      </c>
+      <c r="D27" s="35" t="n"/>
+      <c r="E27" s="35" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="55" t="inlineStr">
+        <is>
+          <t>MEAN (Q19)</t>
+        </is>
+      </c>
+      <c r="D28" s="56">
+        <f>IFERROR(AVERAGEIF(D19:D27,"&lt;&gt;"),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: Apply table row formatting to new participants P10-P12 in SUS workbook
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/research/SUS_Evaluation_IPDC_OSS.xlsx
+++ b/data/research/SUS_Evaluation_IPDC_OSS.xlsx
@@ -1004,7 +1004,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1083,7 +1083,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1109,7 +1109,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4706,120 +4706,120 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>Headquarters</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="23" t="inlineStr">
         <is>
           <t>Laptop (Chrome)</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="23" t="inlineStr">
         <is>
           <t>18 Mar 2026</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="13" ht="14.5" customHeight="1" s="54">
-      <c r="A13" s="82" t="n">
+      <c r="A13" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>Headquarters</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="23" t="inlineStr">
         <is>
           <t>Laptop (Chrome)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="23" t="inlineStr">
         <is>
           <t>18 Mar 2026</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>Tenant Representative</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="23" t="inlineStr">
         <is>
           <t>Kilinto SEZ</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="23" t="inlineStr">
         <is>
           <t>Smartphone (Chrome)</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="23" t="inlineStr">
         <is>
           <t>22 Mar 2026</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="23" t="inlineStr">
         <is>
           <t>Foreign-invested</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="23" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
@@ -6394,137 +6394,137 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="29" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J14" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K14" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L14" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" s="30" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" s="54">
-      <c r="A15" s="79" t="n">
+      <c r="A15" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="29" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="J15" t="n">
+      <c r="J15" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="K15" t="n">
+      <c r="K15" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L15" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="M15" t="n">
+      <c r="M15" s="30" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="29" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="23" t="inlineStr">
         <is>
           <t>Tenant Representative</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H16" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J16" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L16" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" s="30" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8261,201 +8261,214 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D13">
+      <c r="D13" s="30">
         <f>IF('SUS Raw Responses'!D14="","",'SUS Raw Responses'!D14-1)</f>
         <v/>
       </c>
-      <c r="E13">
+      <c r="E13" s="37">
         <f>IF('SUS Raw Responses'!E14="","",5-'SUS Raw Responses'!E14)</f>
         <v/>
       </c>
-      <c r="F13">
+      <c r="F13" s="30">
         <f>IF('SUS Raw Responses'!F14="","",'SUS Raw Responses'!F14-1)</f>
         <v/>
       </c>
-      <c r="G13">
+      <c r="G13" s="37">
         <f>IF('SUS Raw Responses'!G14="","",5-'SUS Raw Responses'!G14)</f>
         <v/>
       </c>
-      <c r="H13">
+      <c r="H13" s="30">
         <f>IF('SUS Raw Responses'!H14="","",'SUS Raw Responses'!H14-1)</f>
         <v/>
       </c>
-      <c r="I13">
+      <c r="I13" s="37">
         <f>IF('SUS Raw Responses'!I14="","",5-'SUS Raw Responses'!I14)</f>
         <v/>
       </c>
-      <c r="J13">
+      <c r="J13" s="30">
         <f>IF('SUS Raw Responses'!J14="","",'SUS Raw Responses'!J14-1)</f>
         <v/>
       </c>
-      <c r="K13">
+      <c r="K13" s="37">
         <f>IF('SUS Raw Responses'!K14="","",5-'SUS Raw Responses'!K14)</f>
         <v/>
       </c>
-      <c r="L13">
+      <c r="L13" s="30">
         <f>IF('SUS Raw Responses'!L14="","",'SUS Raw Responses'!L14-1)</f>
         <v/>
       </c>
-      <c r="M13">
+      <c r="M13" s="37">
         <f>IF('SUS Raw Responses'!M14="","",5-'SUS Raw Responses'!M14)</f>
         <v/>
       </c>
-      <c r="N13">
+      <c r="N13" s="38">
         <f>IF(COUNTA(D13,E13,F13,G13,H13,I13,J13,K13,L13,M13)=10,SUM(D13,E13,F13,G13,H13,I13,J13,K13,L13,M13),"")</f>
         <v/>
       </c>
-      <c r="O13">
+      <c r="O13" s="39">
         <f>IF(N13="","",N13*2.5)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" s="54">
-      <c r="A14" s="45" t="n">
+      <c r="A14" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="29" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D14">
+      <c r="D14" s="30">
         <f>IF('SUS Raw Responses'!D15="","",'SUS Raw Responses'!D15-1)</f>
         <v/>
       </c>
-      <c r="E14">
+      <c r="E14" s="37">
         <f>IF('SUS Raw Responses'!E15="","",5-'SUS Raw Responses'!E15)</f>
         <v/>
       </c>
-      <c r="F14">
+      <c r="F14" s="30">
         <f>IF('SUS Raw Responses'!F15="","",'SUS Raw Responses'!F15-1)</f>
         <v/>
       </c>
-      <c r="G14">
+      <c r="G14" s="37">
         <f>IF('SUS Raw Responses'!G15="","",5-'SUS Raw Responses'!G15)</f>
         <v/>
       </c>
-      <c r="H14">
+      <c r="H14" s="30">
         <f>IF('SUS Raw Responses'!H15="","",'SUS Raw Responses'!H15-1)</f>
         <v/>
       </c>
-      <c r="I14">
+      <c r="I14" s="37">
         <f>IF('SUS Raw Responses'!I15="","",5-'SUS Raw Responses'!I15)</f>
         <v/>
       </c>
-      <c r="J14">
+      <c r="J14" s="30">
         <f>IF('SUS Raw Responses'!J15="","",'SUS Raw Responses'!J15-1)</f>
         <v/>
       </c>
-      <c r="K14">
+      <c r="K14" s="37">
         <f>IF('SUS Raw Responses'!K15="","",5-'SUS Raw Responses'!K15)</f>
         <v/>
       </c>
-      <c r="L14">
+      <c r="L14" s="30">
         <f>IF('SUS Raw Responses'!L15="","",'SUS Raw Responses'!L15-1)</f>
         <v/>
       </c>
-      <c r="M14">
+      <c r="M14" s="37">
         <f>IF('SUS Raw Responses'!M15="","",5-'SUS Raw Responses'!M15)</f>
         <v/>
       </c>
-      <c r="N14">
+      <c r="N14" s="38">
         <f>IF(COUNTA(D14,E14,F14,G14,H14,I14,J14,K14,L14,M14)=10,SUM(D14,E14,F14,G14,H14,I14,J14,K14,L14,M14),"")</f>
         <v/>
       </c>
-      <c r="O14" s="42">
+      <c r="O14" s="39">
         <f>IF(N14="","",N14*2.5)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="29" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>Tenant Representative</t>
         </is>
       </c>
-      <c r="D15">
+      <c r="D15" s="30">
         <f>IF('SUS Raw Responses'!D16="","",'SUS Raw Responses'!D16-1)</f>
         <v/>
       </c>
-      <c r="E15">
+      <c r="E15" s="37">
         <f>IF('SUS Raw Responses'!E16="","",5-'SUS Raw Responses'!E16)</f>
         <v/>
       </c>
-      <c r="F15">
+      <c r="F15" s="30">
         <f>IF('SUS Raw Responses'!F16="","",'SUS Raw Responses'!F16-1)</f>
         <v/>
       </c>
-      <c r="G15">
+      <c r="G15" s="37">
         <f>IF('SUS Raw Responses'!G16="","",5-'SUS Raw Responses'!G16)</f>
         <v/>
       </c>
-      <c r="H15">
+      <c r="H15" s="30">
         <f>IF('SUS Raw Responses'!H16="","",'SUS Raw Responses'!H16-1)</f>
         <v/>
       </c>
-      <c r="I15">
+      <c r="I15" s="37">
         <f>IF('SUS Raw Responses'!I16="","",5-'SUS Raw Responses'!I16)</f>
         <v/>
       </c>
-      <c r="J15">
+      <c r="J15" s="30">
         <f>IF('SUS Raw Responses'!J16="","",'SUS Raw Responses'!J16-1)</f>
         <v/>
       </c>
-      <c r="K15">
+      <c r="K15" s="37">
         <f>IF('SUS Raw Responses'!K16="","",5-'SUS Raw Responses'!K16)</f>
         <v/>
       </c>
-      <c r="L15">
+      <c r="L15" s="30">
         <f>IF('SUS Raw Responses'!L16="","",'SUS Raw Responses'!L16-1)</f>
         <v/>
       </c>
-      <c r="M15">
+      <c r="M15" s="37">
         <f>IF('SUS Raw Responses'!M16="","",5-'SUS Raw Responses'!M16)</f>
         <v/>
       </c>
-      <c r="N15">
+      <c r="N15" s="38">
         <f>IF(COUNTA(D15,E15,F15,G15,H15,I15,J15,K15,L15,M15)=10,SUM(D15,E15,F15,G15,H15,I15,J15,K15,L15,M15),"")</f>
         <v/>
       </c>
-      <c r="O15">
+      <c r="O15" s="39">
         <f>IF(N15="","",N15*2.5)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>MEAN SUS SCORE</t>
         </is>
       </c>
-      <c r="O16">
+      <c r="B16" s="29" t="n"/>
+      <c r="C16" s="23" t="n"/>
+      <c r="D16" s="30" t="n"/>
+      <c r="E16" s="37" t="n"/>
+      <c r="F16" s="30" t="n"/>
+      <c r="G16" s="37" t="n"/>
+      <c r="H16" s="30" t="n"/>
+      <c r="I16" s="37" t="n"/>
+      <c r="J16" s="30" t="n"/>
+      <c r="K16" s="37" t="n"/>
+      <c r="L16" s="30" t="n"/>
+      <c r="M16" s="37" t="n"/>
+      <c r="N16" s="38" t="n"/>
+      <c r="O16" s="39">
         <f>IF(COUNTA(O4:O15)=12,AVERAGE(O4:O15),"")</f>
         <v/>
       </c>
@@ -9442,10 +9455,10 @@
     <row r="1000" ht="15.75" customHeight="1" s="54"/>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="C2:C3"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -9804,116 +9817,119 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="29" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>Laptop (Chrome)</t>
         </is>
       </c>
-      <c r="E12">
+      <c r="E12" s="43">
         <f>'SUS Score Calculation'!O13</f>
         <v/>
       </c>
-      <c r="F12">
+      <c r="F12" s="30">
         <f>IF(E12="","",IF(E12&gt;85.5,"A",IF(E12&gt;=72.6,"B",IF(E12&gt;=52,"C",IF(E12&gt;=51.7,"D","F")))))</f>
         <v/>
       </c>
-      <c r="G12">
+      <c r="G12" s="23">
         <f>IF(E12="","",IF(E12&gt;85.5,"Excellent",IF(E12&gt;=72.6,"Good",IF(E12&gt;=52,"OK",IF(E12&gt;=51.7,"Poor","Awful")))))</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="25.5" customHeight="1" s="54">
-      <c r="A13" s="45" t="n">
+      <c r="A13" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>Laptop (Chrome)</t>
         </is>
       </c>
-      <c r="E13" s="42">
+      <c r="E13" s="43">
         <f>'SUS Score Calculation'!O14</f>
         <v/>
       </c>
-      <c r="F13" s="44">
+      <c r="F13" s="30">
         <f>IF(E13="","",IF(E13&gt;85.5,"A",IF(E13&gt;=72.6,"B",IF(E13&gt;=52,"C",IF(E13&gt;=51.7,"D","F")))))</f>
         <v/>
       </c>
-      <c r="G13" s="45">
+      <c r="G13" s="23">
         <f>IF(E13="","",IF(E13&gt;85.5,"Excellent",IF(E13&gt;=72.6,"Good",IF(E13&gt;=52,"OK",IF(E13&gt;=51.7,"Poor","Awful")))))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="29" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>Tenant Representative</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="23" t="inlineStr">
         <is>
           <t>Smartphone (Chrome)</t>
         </is>
       </c>
-      <c r="E14">
+      <c r="E14" s="43">
         <f>'SUS Score Calculation'!O15</f>
         <v/>
       </c>
-      <c r="F14">
+      <c r="F14" s="30">
         <f>IF(E14="","",IF(E14&gt;85.5,"A",IF(E14&gt;=72.6,"B",IF(E14&gt;=52,"C",IF(E14&gt;=51.7,"D","F")))))</f>
         <v/>
       </c>
-      <c r="G14">
+      <c r="G14" s="23">
         <f>IF(E14="","",IF(E14&gt;85.5,"Excellent",IF(E14&gt;=72.6,"Good",IF(E14&gt;=52,"OK",IF(E14&gt;=51.7,"Poor","Awful")))))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>MEAN SUS SCORE</t>
         </is>
       </c>
-      <c r="E15">
+      <c r="B15" s="29" t="n"/>
+      <c r="C15" s="23" t="n"/>
+      <c r="D15" s="23" t="n"/>
+      <c r="E15" s="43">
         <f>AVERAGE(E3:E14)</f>
         <v/>
       </c>
-      <c r="F15">
+      <c r="F15" s="30">
         <f>IF(E15="","",IF(E15&gt;85.5,"A",IF(E15&gt;=72.6,"B",IF(E15&gt;=52,"C",IF(E15&gt;=51.7,"D","F")))))</f>
         <v/>
       </c>
-      <c r="G15">
+      <c r="G15" s="23">
         <f>IF(E15="","",IF(E15&gt;85.5,"Excellent",IF(E15&gt;=72.6,"Good",IF(E15&gt;=52,"OK",IF(E15&gt;=51.7,"Poor","Awful")))))</f>
         <v/>
       </c>
@@ -10907,8 +10923,8 @@
     <row r="1000" ht="15.75" customHeight="1" s="54"/>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A16:G16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -11278,75 +11294,87 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="D14" s="46" t="n"/>
+      <c r="E14" s="46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F14" s="46" t="n"/>
+      <c r="G14" s="46" t="n"/>
+      <c r="H14" s="46" t="n"/>
+      <c r="I14" s="46" t="n"/>
     </row>
     <row r="15" ht="14.5" customHeight="1" s="54">
-      <c r="A15" s="82" t="n">
+      <c r="A15" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="D15" s="46" t="n"/>
+      <c r="E15" s="46" t="n"/>
+      <c r="F15" s="46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G15" s="46" t="n"/>
+      <c r="H15" s="46" t="n"/>
+      <c r="I15" s="46" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="23" t="inlineStr">
         <is>
           <t>Tenant Representative</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="F16" s="46" t="n"/>
+      <c r="G16" s="46" t="n"/>
+      <c r="H16" s="46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -11713,12 +11741,12 @@
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="54">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="89" t="inlineStr">
         <is>
           <t>MEAN (Q19)</t>
         </is>
       </c>
-      <c r="D33">
+      <c r="D33" s="47">
         <f>IFERROR(AVERAGEIF(D21:D32,"&lt;&gt;"),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fix: Update actual participant roles and devices for P1-P9 across all sheets
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/research/SUS_Evaluation_IPDC_OSS.xlsx
+++ b/data/research/SUS_Evaluation_IPDC_OSS.xlsx
@@ -7767,7 +7767,7 @@
       </c>
       <c r="C5" s="24" t="inlineStr">
         <is>
-          <t>IPDC Management Staff</t>
+          <t>Tenant Representative</t>
         </is>
       </c>
       <c r="D5" s="40">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="C7" s="24" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D7" s="40">
@@ -7956,7 +7956,7 @@
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>IPDC Management Staff</t>
         </is>
       </c>
       <c r="D8" s="30">
@@ -8019,7 +8019,7 @@
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D9" s="40">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Operations Staff</t>
+          <t>Tenant Representative</t>
         </is>
       </c>
       <c r="D12" s="30">
@@ -9544,7 +9544,7 @@
       </c>
       <c r="D3" s="23" t="inlineStr">
         <is>
-          <t>Laptop (Chrome)</t>
+          <t>Smartphone (Chrome)</t>
         </is>
       </c>
       <c r="E3" s="43">
@@ -9571,12 +9571,12 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
-          <t>IPDC Management Staff</t>
+          <t>Tenant Representative</t>
         </is>
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>Desktop (Chrome)</t>
+          <t>Desktop Computer ( Opera)</t>
         </is>
       </c>
       <c r="E4" s="43">
@@ -9608,7 +9608,7 @@
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>Laptop (Opera)</t>
+          <t>Laptop (Chrome)</t>
         </is>
       </c>
       <c r="E5" s="43">
@@ -9635,12 +9635,12 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>Smartphone (Chrome)</t>
+          <t>Laptop (Chrome)</t>
         </is>
       </c>
       <c r="E6" s="43">
@@ -9667,12 +9667,12 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>IPDC Management Staff</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Smartphone (Opera)</t>
+          <t>Laptop (Chrome)</t>
         </is>
       </c>
       <c r="E7" s="43">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>Tenant Representative</t>
+          <t>Operations Staff</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
@@ -9736,7 +9736,7 @@
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Smartphone (Chrome)</t>
+          <t>Laptop (Chrome)</t>
         </is>
       </c>
       <c r="E9" s="43">
@@ -9768,7 +9768,7 @@
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>Smartphone (Opera)</t>
+          <t>Desktop Computer (Chrome)</t>
         </is>
       </c>
       <c r="E10" s="43">
@@ -9795,12 +9795,12 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Operations Staff</t>
+          <t>Tenant Representative</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Smartphone (Chrome)</t>
+          <t>Smartphone (Opera)</t>
         </is>
       </c>
       <c r="E11" s="43">

</xml_diff>

<commit_message>
Fix: Clean up all sheet formatting, update header dates, fix P12 date to 18 Mar 2026
- Updated Participant Profiles header to '9-18 March 2026 | 12 Participants'
- Changed P12 date from 22 Mar to 18 Mar 2026 across all sheets
- Rebuilt Offline Experience Q19/Q20 section cleanly (removed stale rows)
- Fixed P11/P12 row styles in SUS Score Calculation and Summary & Results

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/research/SUS_Evaluation_IPDC_OSS.xlsx
+++ b/data/research/SUS_Evaluation_IPDC_OSS.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -203,6 +203,10 @@
       <color rgb="FF2E7D32"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font/>
   </fonts>
   <fills count="14">
     <fill>
@@ -284,7 +288,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -431,11 +435,12 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -680,6 +685,11 @@
     <xf numFmtId="0" fontId="18" fillId="13" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4299,7 +4309,7 @@
     <row r="1" ht="31.5" customHeight="1" s="54">
       <c r="A1" s="81" t="inlineStr">
         <is>
-          <t>Usability Evaluation — Participant Profiles (10 February 2026)</t>
+          <t>Usability Evaluation — Participant Profiles (9–18 March 2026 | 12 Participants | Chapter 5)</t>
         </is>
       </c>
     </row>
@@ -4811,7 +4821,7 @@
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>22 Mar 2026</t>
+          <t>18 Mar 2026</t>
         </is>
       </c>
       <c r="G14" s="23" t="inlineStr">
@@ -7534,7 +7544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="54" min="1" max="2"/>
@@ -8385,6 +8395,7 @@
         <f>IF(N14="","",N14*2.5)</f>
         <v/>
       </c>
+      <c r="P14" s="90" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="23" t="n">
@@ -8448,9 +8459,11 @@
         <f>IF(N15="","",N15*2.5)</f>
         <v/>
       </c>
+      <c r="P15" s="90" t="n"/>
+      <c r="Q15" s="90" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="91" t="inlineStr">
         <is>
           <t>MEAN SUS SCORE</t>
         </is>
@@ -8472,6 +8485,9 @@
         <f>IF(COUNTA(O4:O15)=12,AVERAGE(O4:O15),"")</f>
         <v/>
       </c>
+      <c r="P16" s="90" t="n"/>
+      <c r="Q16" s="90" t="n"/>
+      <c r="R16" s="90" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="54"/>
     <row r="22" ht="15.75" customHeight="1" s="54"/>
@@ -9471,7 +9487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="54" min="1" max="1"/>
@@ -9879,6 +9895,7 @@
         <f>IF(E13="","",IF(E13&gt;85.5,"Excellent",IF(E13&gt;=72.6,"Good",IF(E13&gt;=52,"OK",IF(E13&gt;=51.7,"Poor","Awful")))))</f>
         <v/>
       </c>
+      <c r="H13" s="90" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="23" t="n">
@@ -9911,9 +9928,11 @@
         <f>IF(E14="","",IF(E14&gt;85.5,"Excellent",IF(E14&gt;=72.6,"Good",IF(E14&gt;=52,"OK",IF(E14&gt;=51.7,"Poor","Awful")))))</f>
         <v/>
       </c>
+      <c r="H14" s="90" t="n"/>
+      <c r="I14" s="90" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="91" t="inlineStr">
         <is>
           <t>MEAN SUS SCORE</t>
         </is>
@@ -9933,6 +9952,9 @@
         <f>IF(E15="","",IF(E15&gt;85.5,"Excellent",IF(E15&gt;=72.6,"Good",IF(E15&gt;=52,"OK",IF(E15&gt;=51.7,"Poor","Awful")))))</f>
         <v/>
       </c>
+      <c r="H15" s="90" t="n"/>
+      <c r="I15" s="90" t="n"/>
+      <c r="J15" s="90" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="54">
       <c r="A16" s="86" t="inlineStr">
@@ -10938,7 +10960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6" customWidth="1" style="54" min="1" max="1"/>
@@ -11381,88 +11403,84 @@
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" s="54">
-      <c r="A17" s="88" t="inlineStr">
+      <c r="A17" s="87" t="inlineStr">
         <is>
           <t>Enter  ✓  if the participant attempted the task, or leave blank if not attempted.</t>
         </is>
       </c>
+      <c r="B17" s="90" t="n"/>
+      <c r="C17" s="90" t="n"/>
+      <c r="D17" s="90" t="n"/>
+      <c r="E17" s="90" t="n"/>
+      <c r="F17" s="90" t="n"/>
+      <c r="G17" s="90" t="n"/>
+      <c r="H17" s="90" t="n"/>
+      <c r="I17" s="90" t="n"/>
+      <c r="J17" s="90" t="n"/>
     </row>
     <row r="18" ht="43.5" customHeight="1" s="54">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="92" t="n"/>
+      <c r="B18" s="92" t="n"/>
+      <c r="C18" s="92" t="n"/>
+      <c r="D18" s="92" t="n"/>
+      <c r="E18" s="92" t="n"/>
+      <c r="F18" s="92" t="n"/>
+      <c r="G18" s="92" t="n"/>
+      <c r="H18" s="92" t="n"/>
+      <c r="I18" s="92" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="54">
+      <c r="A19" s="88" t="inlineStr">
+        <is>
+          <t>Q19 — Offline Confidence Score  |  Q20 — Online/Offline Clarity  |  Google Form: Section 8 of 9</t>
+        </is>
+      </c>
+      <c r="B19" s="90" t="n"/>
+      <c r="C19" s="90" t="n"/>
+      <c r="D19" s="90" t="n"/>
+      <c r="E19" s="90" t="n"/>
+      <c r="F19" s="90" t="n"/>
+      <c r="G19" s="90" t="n"/>
+      <c r="H19" s="90" t="n"/>
+      <c r="I19" s="90" t="n"/>
+      <c r="J19" s="90" t="n"/>
+      <c r="K19" s="90" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="54">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B18" s="32" t="inlineStr">
+      <c r="B20" s="32" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C18" s="32" t="inlineStr">
+      <c r="C20" s="32" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="D18" s="32" t="inlineStr">
+      <c r="D20" s="32" t="inlineStr">
         <is>
           <t>Q19: Offline data confidence (1–5)
 1=Not confident  5=Fully confident</t>
         </is>
       </c>
-      <c r="E18" s="32" t="inlineStr">
+      <c r="E20" s="32" t="inlineStr">
         <is>
           <t>Q20: Online/offline clarity
 Yes always / Sometimes / No</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="18" customHeight="1" s="54">
-      <c r="A19" s="23" t="inlineStr">
-        <is>
-          <t>Q19 — Offline Confidence Score  |  Q20 — Online/Offline Clarity  |  Google Form: Section 8 of 9</t>
-        </is>
-      </c>
-      <c r="B19" s="23" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="inlineStr">
-        <is>
-          <t>IPDC Management Staff</t>
-        </is>
-      </c>
-      <c r="D19" s="30" t="n"/>
-      <c r="E19" s="30" t="n"/>
-    </row>
-    <row r="20" ht="18" customHeight="1" s="54">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B20" s="24" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="C20" s="24" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="D20" s="30" t="inlineStr">
-        <is>
-          <t>Q19: Offline data confidence (1–5)
-1=Not confident  5=Fully confident</t>
-        </is>
-      </c>
-      <c r="E20" s="30" t="inlineStr">
-        <is>
-          <t>Q20: Online/offline clarity
-Yes always / Sometimes / No</t>
-        </is>
-      </c>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+      <c r="J20" s="90" t="n"/>
+      <c r="K20" s="90" t="n"/>
+      <c r="L20" s="90" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1" s="54">
       <c r="A21" s="23" t="n">
@@ -11626,130 +11644,196 @@
       </c>
     </row>
     <row r="28" ht="21.75" customHeight="1" s="54">
-      <c r="A28" s="89" t="n">
+      <c r="A28" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D28" s="47" t="n">
+      <c r="D28" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="30" t="inlineStr">
         <is>
           <t>Yes, it was always clear</t>
         </is>
       </c>
+      <c r="F28" s="90" t="n"/>
+      <c r="G28" s="90" t="n"/>
+      <c r="H28" s="90" t="n"/>
+      <c r="I28" s="90" t="n"/>
+      <c r="J28" s="90" t="n"/>
+      <c r="K28" s="90" t="n"/>
+      <c r="L28" s="90" t="n"/>
+      <c r="M28" s="90" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="54">
-      <c r="A29" t="n">
+      <c r="A29" s="23" t="n">
         <v>9</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>P9</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="23" t="inlineStr">
         <is>
           <t>Tenant Representative</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="30" t="inlineStr">
         <is>
           <t>Yes, it was always clear</t>
         </is>
       </c>
+      <c r="F29" s="90" t="n"/>
+      <c r="G29" s="90" t="n"/>
+      <c r="H29" s="90" t="n"/>
+      <c r="I29" s="90" t="n"/>
+      <c r="J29" s="90" t="n"/>
+      <c r="K29" s="90" t="n"/>
+      <c r="L29" s="90" t="n"/>
+      <c r="M29" s="90" t="n"/>
+      <c r="N29" s="90" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="54">
-      <c r="A30" t="n">
+      <c r="A30" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="23" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D30" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="30" t="inlineStr">
         <is>
           <t>Sometimes clear, sometimes not</t>
         </is>
       </c>
+      <c r="F30" s="90" t="n"/>
+      <c r="G30" s="90" t="n"/>
+      <c r="H30" s="90" t="n"/>
+      <c r="I30" s="90" t="n"/>
+      <c r="J30" s="90" t="n"/>
+      <c r="K30" s="90" t="n"/>
+      <c r="L30" s="90" t="n"/>
+      <c r="M30" s="90" t="n"/>
+      <c r="N30" s="90" t="n"/>
+      <c r="O30" s="90" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="54">
-      <c r="A31" t="n">
+      <c r="A31" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="23" t="inlineStr">
         <is>
           <t>Operations Staff</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="30" t="inlineStr">
         <is>
           <t>Yes, it was always clear</t>
         </is>
       </c>
+      <c r="F31" s="90" t="n"/>
+      <c r="G31" s="90" t="n"/>
+      <c r="H31" s="90" t="n"/>
+      <c r="I31" s="90" t="n"/>
+      <c r="J31" s="90" t="n"/>
+      <c r="K31" s="90" t="n"/>
+      <c r="L31" s="90" t="n"/>
+      <c r="M31" s="90" t="n"/>
+      <c r="N31" s="90" t="n"/>
+      <c r="O31" s="90" t="n"/>
+      <c r="P31" s="90" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="54">
-      <c r="A32" t="n">
+      <c r="A32" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="23" t="inlineStr">
         <is>
           <t>Tenant Representative</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="30" t="inlineStr">
         <is>
           <t>Yes, it was always clear</t>
         </is>
       </c>
+      <c r="F32" s="90" t="n"/>
+      <c r="G32" s="90" t="n"/>
+      <c r="H32" s="90" t="n"/>
+      <c r="I32" s="90" t="n"/>
+      <c r="J32" s="90" t="n"/>
+      <c r="K32" s="90" t="n"/>
+      <c r="L32" s="90" t="n"/>
+      <c r="M32" s="90" t="n"/>
+      <c r="N32" s="90" t="n"/>
+      <c r="O32" s="90" t="n"/>
+      <c r="P32" s="90" t="n"/>
+      <c r="Q32" s="90" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="54">
-      <c r="A33" s="89" t="inlineStr">
+      <c r="A33" s="91" t="inlineStr">
         <is>
           <t>MEAN (Q19)</t>
         </is>
       </c>
-      <c r="D33" s="47">
+      <c r="B33" s="23" t="n"/>
+      <c r="C33" s="23" t="n"/>
+      <c r="D33" s="30">
         <f>IFERROR(AVERAGEIF(D21:D32,"&lt;&gt;"),"")</f>
         <v/>
       </c>
+      <c r="E33" s="30" t="n"/>
+      <c r="F33" s="90" t="n"/>
+      <c r="G33" s="90" t="n"/>
+      <c r="H33" s="90" t="n"/>
+      <c r="I33" s="90" t="n"/>
+      <c r="J33" s="90" t="n"/>
+      <c r="K33" s="90" t="n"/>
+      <c r="L33" s="90" t="n"/>
+      <c r="M33" s="90" t="n"/>
+      <c r="N33" s="90" t="n"/>
+      <c r="O33" s="90" t="n"/>
+      <c r="P33" s="90" t="n"/>
+      <c r="Q33" s="90" t="n"/>
+      <c r="R33" s="90" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="54"/>
     <row r="35" ht="15.75" customHeight="1" s="54"/>

</xml_diff>

<commit_message>
Fix: Widen all columns so text is fully visible across all sheets
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/research/SUS_Evaluation_IPDC_OSS.xlsx
+++ b/data/research/SUS_Evaluation_IPDC_OSS.xlsx
@@ -1399,26 +1399,34 @@
   <dimension ref="A1:AB13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="21.6328125" customWidth="1" style="54" min="1" max="1"/>
-    <col width="32" customWidth="1" style="54" min="2" max="2"/>
-    <col width="43" customWidth="1" style="54" min="3" max="5"/>
-    <col width="24" customWidth="1" style="54" min="6" max="6"/>
-    <col width="24.26953125" customWidth="1" style="54" min="7" max="7"/>
-    <col width="23.453125" customWidth="1" style="54" min="8" max="8"/>
-    <col width="53.7265625" customWidth="1" style="54" min="9" max="9"/>
-    <col width="52.90625" customWidth="1" style="54" min="10" max="10"/>
-    <col width="43" customWidth="1" style="54" min="11" max="16"/>
-    <col width="59.54296875" customWidth="1" style="54" min="17" max="17"/>
-    <col width="43" customWidth="1" style="54" min="18" max="18"/>
-    <col width="71.81640625" customWidth="1" style="54" min="19" max="19"/>
-    <col width="43" customWidth="1" style="54" min="20" max="21"/>
-    <col width="57.1796875" customWidth="1" style="54" min="22" max="22"/>
-    <col width="49.453125" customWidth="1" style="54" min="23" max="23"/>
-    <col width="43" customWidth="1" style="54" min="24" max="24"/>
-    <col width="110.26953125" customWidth="1" style="54" min="25" max="25"/>
-    <col width="86.1796875" customWidth="1" style="54" min="26" max="26"/>
-    <col width="59.90625" customWidth="1" style="54" min="27" max="27"/>
-    <col width="65.6328125" customWidth="1" style="54" min="28" max="28"/>
+    <col width="28" customWidth="1" style="54" min="1" max="1"/>
+    <col width="45" customWidth="1" style="54" min="2" max="2"/>
+    <col width="45" customWidth="1" style="54" min="3" max="5"/>
+    <col width="45" customWidth="1" style="54" min="4" max="4"/>
+    <col width="45" customWidth="1" style="54" min="5" max="5"/>
+    <col width="18" customWidth="1" style="54" min="6" max="6"/>
+    <col width="30" customWidth="1" style="54" min="7" max="7"/>
+    <col width="21" customWidth="1" style="54" min="8" max="8"/>
+    <col width="45" customWidth="1" style="54" min="9" max="9"/>
+    <col width="45" customWidth="1" style="54" min="10" max="10"/>
+    <col width="45" customWidth="1" style="54" min="11" max="16"/>
+    <col width="45" customWidth="1" style="54" min="12" max="12"/>
+    <col width="45" customWidth="1" style="54" min="13" max="13"/>
+    <col width="45" customWidth="1" style="54" min="14" max="14"/>
+    <col width="45" customWidth="1" style="54" min="15" max="15"/>
+    <col width="45" customWidth="1" style="54" min="16" max="16"/>
+    <col width="45" customWidth="1" style="54" min="17" max="17"/>
+    <col width="45" customWidth="1" style="54" min="18" max="18"/>
+    <col width="45" customWidth="1" style="54" min="19" max="19"/>
+    <col width="45" customWidth="1" style="54" min="20" max="21"/>
+    <col width="45" customWidth="1" style="54" min="21" max="21"/>
+    <col width="45" customWidth="1" style="54" min="22" max="22"/>
+    <col width="45" customWidth="1" style="54" min="23" max="23"/>
+    <col width="45" customWidth="1" style="54" min="24" max="24"/>
+    <col width="45" customWidth="1" style="54" min="25" max="25"/>
+    <col width="45" customWidth="1" style="54" min="26" max="26"/>
+    <col width="45" customWidth="1" style="54" min="27" max="27"/>
+    <col width="45" customWidth="1" style="54" min="28" max="28"/>
     <col width="21.54296875" customWidth="1" style="54" min="29" max="34"/>
   </cols>
   <sheetData>
@@ -2744,10 +2752,10 @@
   <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="4" customWidth="1" style="54" min="1" max="1"/>
-    <col width="28" customWidth="1" style="54" min="2" max="2"/>
-    <col width="70" customWidth="1" style="54" min="3" max="3"/>
-    <col width="20" customWidth="1" style="54" min="4" max="4"/>
+    <col width="45" customWidth="1" style="54" min="1" max="1"/>
+    <col width="42" customWidth="1" style="54" min="2" max="2"/>
+    <col width="45" customWidth="1" style="54" min="3" max="3"/>
+    <col width="45" customWidth="1" style="54" min="4" max="4"/>
     <col width="8.7265625" customWidth="1" style="54" min="5" max="26"/>
   </cols>
   <sheetData>
@@ -2765,6 +2773,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="14.5" customHeight="1" s="54">
       <c r="A4" s="74" t="inlineStr">
         <is>
@@ -2779,6 +2788,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="14.5" customHeight="1" s="54">
       <c r="A7" s="74" t="inlineStr">
         <is>
@@ -2864,6 +2874,7 @@
       </c>
       <c r="D13" s="77" t="n"/>
     </row>
+    <row r="14"/>
     <row r="15" ht="14.5" customHeight="1" s="54">
       <c r="A15" s="74" t="inlineStr">
         <is>
@@ -2923,6 +2934,7 @@
       </c>
       <c r="D19" s="77" t="n"/>
     </row>
+    <row r="20"/>
     <row r="21" ht="15.75" customHeight="1" s="54">
       <c r="A21" s="74" t="inlineStr">
         <is>
@@ -4296,13 +4308,14 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="6" customWidth="1" style="54" min="1" max="1"/>
-    <col width="8" customWidth="1" style="54" min="2" max="2"/>
-    <col width="28" customWidth="1" style="54" min="3" max="3"/>
-    <col width="22" customWidth="1" style="54" min="4" max="4"/>
-    <col width="20" customWidth="1" style="54" min="5" max="5"/>
-    <col width="16" customWidth="1" style="54" min="6" max="6"/>
-    <col width="20" customWidth="1" style="54" min="7" max="8"/>
+    <col width="45" customWidth="1" style="54" min="1" max="1"/>
+    <col width="10" customWidth="1" style="54" min="2" max="2"/>
+    <col width="23" customWidth="1" style="54" min="3" max="3"/>
+    <col width="23" customWidth="1" style="54" min="4" max="4"/>
+    <col width="27" customWidth="1" style="54" min="5" max="5"/>
+    <col width="13" customWidth="1" style="54" min="6" max="6"/>
+    <col width="19" customWidth="1" style="54" min="7" max="8"/>
+    <col width="19" customWidth="1" style="54" min="8" max="8"/>
     <col width="8.7265625" customWidth="1" style="54" min="9" max="26"/>
   </cols>
   <sheetData>
@@ -5840,9 +5853,19 @@
   <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="8" customWidth="1" style="54" min="1" max="2"/>
-    <col width="26" customWidth="1" style="54" min="3" max="3"/>
-    <col width="10" customWidth="1" style="54" min="4" max="13"/>
+    <col width="45" customWidth="1" style="54" min="1" max="2"/>
+    <col width="10" customWidth="1" style="54" min="2" max="2"/>
+    <col width="23" customWidth="1" style="54" min="3" max="3"/>
+    <col width="45" customWidth="1" style="54" min="4" max="13"/>
+    <col width="43" customWidth="1" style="54" min="5" max="5"/>
+    <col width="39" customWidth="1" style="54" min="6" max="6"/>
+    <col width="45" customWidth="1" style="54" min="7" max="7"/>
+    <col width="45" customWidth="1" style="54" min="8" max="8"/>
+    <col width="45" customWidth="1" style="54" min="9" max="9"/>
+    <col width="45" customWidth="1" style="54" min="10" max="10"/>
+    <col width="44" customWidth="1" style="54" min="11" max="11"/>
+    <col width="41" customWidth="1" style="54" min="12" max="12"/>
+    <col width="45" customWidth="1" style="54" min="13" max="13"/>
     <col width="8.7265625" customWidth="1" style="54" min="14" max="26"/>
   </cols>
   <sheetData>
@@ -7547,10 +7570,21 @@
   <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="8" customWidth="1" style="54" min="1" max="2"/>
-    <col width="26" customWidth="1" style="54" min="3" max="3"/>
-    <col width="11" customWidth="1" style="54" min="4" max="13"/>
-    <col width="14" customWidth="1" style="54" min="14" max="15"/>
+    <col width="45" customWidth="1" style="54" min="1" max="2"/>
+    <col width="10" customWidth="1" style="54" min="2" max="2"/>
+    <col width="23" customWidth="1" style="54" min="3" max="3"/>
+    <col width="45" customWidth="1" style="54" min="4" max="13"/>
+    <col width="45" customWidth="1" style="54" min="5" max="5"/>
+    <col width="45" customWidth="1" style="54" min="6" max="6"/>
+    <col width="45" customWidth="1" style="54" min="7" max="7"/>
+    <col width="45" customWidth="1" style="54" min="8" max="8"/>
+    <col width="45" customWidth="1" style="54" min="9" max="9"/>
+    <col width="45" customWidth="1" style="54" min="10" max="10"/>
+    <col width="45" customWidth="1" style="54" min="11" max="11"/>
+    <col width="45" customWidth="1" style="54" min="12" max="12"/>
+    <col width="45" customWidth="1" style="54" min="13" max="13"/>
+    <col width="45" customWidth="1" style="54" min="14" max="15"/>
+    <col width="43" customWidth="1" style="54" min="15" max="15"/>
     <col width="8.7265625" customWidth="1" style="54" min="16" max="26"/>
   </cols>
   <sheetData>
@@ -9490,13 +9524,13 @@
   <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="8" customWidth="1" style="54" min="1" max="1"/>
+    <col width="45" customWidth="1" style="54" min="1" max="1"/>
     <col width="10" customWidth="1" style="54" min="2" max="2"/>
-    <col width="28" customWidth="1" style="54" min="3" max="3"/>
-    <col width="16" customWidth="1" style="54" min="4" max="4"/>
-    <col width="14" customWidth="1" style="54" min="5" max="5"/>
-    <col width="18" customWidth="1" style="54" min="6" max="6"/>
-    <col width="20" customWidth="1" style="54" min="7" max="7"/>
+    <col width="23" customWidth="1" style="54" min="3" max="3"/>
+    <col width="27" customWidth="1" style="54" min="4" max="4"/>
+    <col width="30" customWidth="1" style="54" min="5" max="5"/>
+    <col width="45" customWidth="1" style="54" min="6" max="6"/>
+    <col width="45" customWidth="1" style="54" min="7" max="7"/>
     <col width="8.7265625" customWidth="1" style="54" min="8" max="26"/>
   </cols>
   <sheetData>
@@ -10963,10 +10997,15 @@
   <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="6" customWidth="1" style="54" min="1" max="1"/>
-    <col width="8" customWidth="1" style="54" min="2" max="2"/>
-    <col width="28" customWidth="1" style="54" min="3" max="3"/>
-    <col width="26" customWidth="1" style="54" min="4" max="9"/>
+    <col width="45" customWidth="1" style="54" min="1" max="1"/>
+    <col width="10" customWidth="1" style="54" min="2" max="2"/>
+    <col width="23" customWidth="1" style="54" min="3" max="3"/>
+    <col width="38" customWidth="1" style="54" min="4" max="9"/>
+    <col width="36" customWidth="1" style="54" min="5" max="5"/>
+    <col width="37" customWidth="1" style="54" min="6" max="6"/>
+    <col width="39" customWidth="1" style="54" min="7" max="7"/>
+    <col width="24" customWidth="1" style="54" min="8" max="8"/>
+    <col width="32" customWidth="1" style="54" min="9" max="9"/>
     <col width="8.7265625" customWidth="1" style="54" min="10" max="26"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Fix: Auto-fit row heights so all wrapped text is fully visible across all sheets
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/research/SUS_Evaluation_IPDC_OSS.xlsx
+++ b/data/research/SUS_Evaluation_IPDC_OSS.xlsx
@@ -1430,7 +1430,7 @@
     <col width="21.54296875" customWidth="1" style="54" min="29" max="34"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="54">
+    <row r="1" ht="60" customHeight="1" s="54">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Timestamp</t>
@@ -1582,7 +1582,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1" s="54">
+    <row r="2" ht="90" customHeight="1" s="54">
       <c r="A2" s="5" t="n">
         <v>46090.50363871528</v>
       </c>
@@ -1680,7 +1680,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1" s="54">
+    <row r="3" ht="30" customHeight="1" s="54">
       <c r="A3" s="5" t="n">
         <v>46097.05842277778</v>
       </c>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="AB3" s="48" t="n"/>
     </row>
-    <row r="4" ht="22.5" customHeight="1" s="54">
+    <row r="4" ht="30" customHeight="1" s="54">
       <c r="A4" s="5" t="n">
         <v>46099.23142234953</v>
       </c>
@@ -1877,7 +1877,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1" s="54">
+    <row r="5" ht="30" customHeight="1" s="54">
       <c r="A5" s="5" t="n">
         <v>46099.24636091435</v>
       </c>
@@ -1970,7 +1970,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1" s="54">
+    <row r="6" ht="30" customHeight="1" s="54">
       <c r="A6" s="5" t="n">
         <v>46099.25548753472</v>
       </c>
@@ -2063,7 +2063,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1" s="54">
+    <row r="7" ht="60" customHeight="1" s="54">
       <c r="A7" s="5" t="n">
         <v>46099.25578788194</v>
       </c>
@@ -2156,7 +2156,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1" s="54">
+    <row r="8" ht="105" customHeight="1" s="54">
       <c r="A8" s="5" t="n">
         <v>46099.25783776621</v>
       </c>
@@ -2249,7 +2249,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1" s="54">
+    <row r="9" ht="60" customHeight="1" s="54">
       <c r="A9" s="5" t="n">
         <v>46099.26724091435</v>
       </c>
@@ -2342,7 +2342,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1" s="54">
+    <row r="10" ht="120" customHeight="1" s="54">
       <c r="A10" s="5" t="n">
         <v>46099.2790071875</v>
       </c>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="AB10" s="6" t="n"/>
     </row>
-    <row r="11" ht="22.5" customHeight="1" s="54">
+    <row r="11" ht="30" customHeight="1" s="54">
       <c r="A11" s="5" t="n">
         <v>46099.30596916666</v>
       </c>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1" s="54">
+    <row r="12" ht="30" customHeight="1" s="54">
       <c r="A12" s="5" t="n">
         <v>46099.30711689815</v>
       </c>
@@ -2627,7 +2627,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="22.5" customHeight="1" s="54">
+    <row r="13" ht="90" customHeight="1" s="54">
       <c r="A13" s="5" t="n">
         <v>46103.97938486111</v>
       </c>
@@ -2759,44 +2759,44 @@
     <col width="8.7265625" customWidth="1" style="54" min="5" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" s="54">
+    <row r="1" ht="30" customHeight="1" s="54">
       <c r="A1" s="72" t="inlineStr">
         <is>
           <t>IPDC-OSS Platform — System Usability Scale (SUS) Evaluation Workbook</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1" s="54">
+    <row r="2" ht="30" customHeight="1" s="54">
       <c r="A2" s="73" t="inlineStr">
         <is>
           <t>Usability Evaluation — 10 February 2026 | 9 Participants | Chapter 5</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4" ht="14.5" customHeight="1" s="54">
+    <row r="3" ht="15" customHeight="1" s="54"/>
+    <row r="4" ht="15" customHeight="1" s="54">
       <c r="A4" s="74" t="inlineStr">
         <is>
           <t>PURPOSE</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1" s="54">
+    <row r="5" ht="105" customHeight="1" s="54">
       <c r="A5" s="75" t="inlineStr">
         <is>
           <t>This workbook is the official data collection and calculation instrument for the SUS usability evaluation of the IPDC Digital One-Stop-Service (OSS) platform prototype. It accompanies the thesis: 'Design and Development of a Digital One-Stop-Service Platform for Industrial Parks in Ethiopia'.</t>
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7" ht="14.5" customHeight="1" s="54">
+    <row r="6" ht="15" customHeight="1" s="54"/>
+    <row r="7" ht="15" customHeight="1" s="54">
       <c r="A7" s="74" t="inlineStr">
         <is>
           <t>WORKBOOK STRUCTURE</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" s="54">
+    <row r="8" ht="30" customHeight="1" s="54">
       <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Instructions</t>
@@ -2809,7 +2809,7 @@
       </c>
       <c r="D8" s="77" t="n"/>
     </row>
-    <row r="9" ht="18" customHeight="1" s="54">
+    <row r="9" ht="30" customHeight="1" s="54">
       <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Participant Profiles</t>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="D9" s="77" t="n"/>
     </row>
-    <row r="10" ht="18" customHeight="1" s="54">
+    <row r="10" ht="30" customHeight="1" s="54">
       <c r="B10" s="7" t="inlineStr">
         <is>
           <t>SUS Raw Responses</t>
@@ -2835,7 +2835,7 @@
       </c>
       <c r="D10" s="77" t="n"/>
     </row>
-    <row r="11" ht="18" customHeight="1" s="54">
+    <row r="11" ht="30" customHeight="1" s="54">
       <c r="B11" s="7" t="inlineStr">
         <is>
           <t>SUS Score Calculation</t>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="D11" s="77" t="n"/>
     </row>
-    <row r="12" ht="18" customHeight="1" s="54">
+    <row r="12" ht="30" customHeight="1" s="54">
       <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Summary &amp; Results</t>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="D12" s="77" t="n"/>
     </row>
-    <row r="13" ht="18" customHeight="1" s="54">
+    <row r="13" ht="30" customHeight="1" s="54">
       <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Offline Experience</t>
@@ -2874,15 +2874,15 @@
       </c>
       <c r="D13" s="77" t="n"/>
     </row>
-    <row r="14"/>
-    <row r="15" ht="14.5" customHeight="1" s="54">
+    <row r="14" ht="15" customHeight="1" s="54"/>
+    <row r="15" ht="15" customHeight="1" s="54">
       <c r="A15" s="74" t="inlineStr">
         <is>
           <t>SUS SCORING FORMULA</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="54">
+    <row r="16" ht="15" customHeight="1" s="54">
       <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Odd items — Positive (Q1,Q3,Q5,Q7,Q9):</t>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="D16" s="77" t="n"/>
     </row>
-    <row r="17" ht="18" customHeight="1" s="54">
+    <row r="17" ht="15" customHeight="1" s="54">
       <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Even items — Negative (Q2,Q4,Q6,Q8,Q10):</t>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="D17" s="77" t="n"/>
     </row>
-    <row r="18" ht="18" customHeight="1" s="54">
+    <row r="18" ht="15" customHeight="1" s="54">
       <c r="B18" s="8" t="inlineStr">
         <is>
           <t>SUS Score:</t>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="D18" s="77" t="n"/>
     </row>
-    <row r="19" ht="18" customHeight="1" s="54">
+    <row r="19" ht="15" customHeight="1" s="54">
       <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Scale:</t>
@@ -2934,15 +2934,15 @@
       </c>
       <c r="D19" s="77" t="n"/>
     </row>
-    <row r="20"/>
-    <row r="21" ht="15.75" customHeight="1" s="54">
+    <row r="20" ht="15" customHeight="1" s="54"/>
+    <row r="21" ht="30" customHeight="1" s="54">
       <c r="A21" s="74" t="inlineStr">
         <is>
           <t>SUS SCORE INTERPRETATION (Bangor et al. / Sauro)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1" s="54">
+    <row r="22" ht="15" customHeight="1" s="54">
       <c r="B22" s="9" t="inlineStr">
         <is>
           <t>&gt; 85.5</t>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1" s="54">
+    <row r="23" ht="15" customHeight="1" s="54">
       <c r="B23" s="11" t="inlineStr">
         <is>
           <t>72.6 – 85.5</t>
@@ -2976,7 +2976,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="54">
+    <row r="24" ht="15" customHeight="1" s="54">
       <c r="B24" s="13" t="inlineStr">
         <is>
           <t>52.0 – 72.5</t>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1" s="54">
+    <row r="25" ht="15" customHeight="1" s="54">
       <c r="B25" s="15" t="inlineStr">
         <is>
           <t>51.7 – 51.9</t>
@@ -3010,7 +3010,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1" s="54">
+    <row r="26" ht="15" customHeight="1" s="54">
       <c r="B26" s="17" t="inlineStr">
         <is>
           <t>&lt; 51.6</t>
@@ -3027,15 +3027,15 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="54"/>
-    <row r="28" ht="15.75" customHeight="1" s="54">
+    <row r="27" ht="15" customHeight="1" s="54"/>
+    <row r="28" ht="15" customHeight="1" s="54">
       <c r="A28" s="74" t="inlineStr">
         <is>
           <t>TASK SCENARIOS ADMINISTERED TO PARTICIPANTS</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1" s="54">
+    <row r="29" ht="45" customHeight="1" s="54">
       <c r="B29" s="19" t="inlineStr">
         <is>
           <t>Task M1</t>
@@ -3052,7 +3052,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1" s="54">
+    <row r="30" ht="45" customHeight="1" s="54">
       <c r="B30" s="19" t="inlineStr">
         <is>
           <t>Task M2</t>
@@ -3069,7 +3069,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1" s="54">
+    <row r="31" ht="45" customHeight="1" s="54">
       <c r="B31" s="19" t="inlineStr">
         <is>
           <t>Task M3</t>
@@ -3086,7 +3086,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1" s="54">
+    <row r="32" ht="45" customHeight="1" s="54">
       <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Task M4</t>
@@ -3103,7 +3103,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1" s="54">
+    <row r="33" ht="45" customHeight="1" s="54">
       <c r="B33" s="19" t="inlineStr">
         <is>
           <t>Task T1</t>
@@ -3120,7 +3120,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1" s="54">
+    <row r="34" ht="45" customHeight="1" s="54">
       <c r="B34" s="19" t="inlineStr">
         <is>
           <t>Task T2</t>
@@ -3137,7 +3137,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1" s="54">
+    <row r="35" ht="45" customHeight="1" s="54">
       <c r="B35" s="19" t="inlineStr">
         <is>
           <t>Task T3</t>
@@ -3154,7 +3154,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1" s="54">
+    <row r="36" ht="45" customHeight="1" s="54">
       <c r="B36" s="19" t="inlineStr">
         <is>
           <t>Task T4</t>
@@ -3171,7 +3171,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1" s="54">
+    <row r="37" ht="45" customHeight="1" s="54">
       <c r="B37" s="19" t="inlineStr">
         <is>
           <t>Task O1</t>
@@ -3188,7 +3188,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1" s="54">
+    <row r="38" ht="45" customHeight="1" s="54">
       <c r="B38" s="19" t="inlineStr">
         <is>
           <t>Task O2</t>
@@ -3222,7 +3222,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1" s="54">
+    <row r="40" ht="45" customHeight="1" s="54">
       <c r="B40" s="19" t="inlineStr">
         <is>
           <t>Task O4</t>
@@ -3239,7 +3239,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1" s="54">
+    <row r="41" ht="45" customHeight="1" s="54">
       <c r="B41" s="19" t="inlineStr">
         <is>
           <t>Task X1</t>
@@ -3256,7 +3256,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1" s="54">
+    <row r="42" ht="45" customHeight="1" s="54">
       <c r="B42" s="19" t="inlineStr">
         <is>
           <t>Task X2</t>
@@ -3273,7 +3273,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="30" customHeight="1" s="54">
+    <row r="43" ht="45" customHeight="1" s="54">
       <c r="B43" s="19" t="inlineStr">
         <is>
           <t>Task X3</t>
@@ -3290,7 +3290,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1" s="54">
+    <row r="44" ht="45" customHeight="1" s="54">
       <c r="B44" s="19" t="inlineStr">
         <is>
           <t>Task X4</t>
@@ -3307,8 +3307,8 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="15.75" customHeight="1" s="54"/>
-    <row r="46" ht="36" customHeight="1" s="54">
+    <row r="45" ht="15" customHeight="1" s="54"/>
+    <row r="46" ht="90" customHeight="1" s="54">
       <c r="A46" s="79" t="inlineStr">
         <is>
           <t>⚠  IMPORTANT: Enter REAL participant responses in the 'SUS Raw Responses' sheet. All SUS scores in the thesis must reflect actual collected data. Scores in 'SUS Score Calculation' and 'Summary &amp; Results' update automatically.</t>
@@ -4319,14 +4319,14 @@
     <col width="8.7265625" customWidth="1" style="54" min="9" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" s="54">
+    <row r="1" ht="45" customHeight="1" s="54">
       <c r="A1" s="81" t="inlineStr">
         <is>
           <t>Usability Evaluation — Participant Profiles (9–18 March 2026 | 12 Participants | Chapter 5)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" s="54">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>#</t>
@@ -4368,7 +4368,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" s="54">
+    <row r="3" ht="15" customHeight="1" s="54">
       <c r="A3" s="23" t="n">
         <v>1</v>
       </c>
@@ -4408,7 +4408,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" s="54">
+    <row r="4" ht="15" customHeight="1" s="54">
       <c r="A4" s="24" t="n">
         <v>2</v>
       </c>
@@ -4448,7 +4448,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1" s="54">
+    <row r="5" ht="15" customHeight="1" s="54">
       <c r="A5" s="23" t="n">
         <v>3</v>
       </c>
@@ -4488,7 +4488,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" s="54">
+    <row r="6" ht="15" customHeight="1" s="54">
       <c r="A6" s="24" t="n">
         <v>4</v>
       </c>
@@ -4528,7 +4528,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1" s="54">
+    <row r="7" ht="15" customHeight="1" s="54">
       <c r="A7" s="23" t="n">
         <v>5</v>
       </c>
@@ -4568,7 +4568,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" s="54">
+    <row r="8" ht="15" customHeight="1" s="54">
       <c r="A8" s="24" t="n">
         <v>6</v>
       </c>
@@ -4608,7 +4608,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" s="54">
+    <row r="9" ht="15" customHeight="1" s="54">
       <c r="A9" s="23" t="n">
         <v>7</v>
       </c>
@@ -4648,7 +4648,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="54">
+    <row r="10" ht="15" customHeight="1" s="54">
       <c r="A10" s="24" t="n">
         <v>8</v>
       </c>
@@ -4688,7 +4688,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" s="54">
+    <row r="11" ht="15" customHeight="1" s="54">
       <c r="A11" s="23" t="n">
         <v>9</v>
       </c>
@@ -4728,7 +4728,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="15" customHeight="1" s="54">
       <c r="A12" s="23" t="n">
         <v>10</v>
       </c>
@@ -4768,7 +4768,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="14.5" customHeight="1" s="54">
+    <row r="13" ht="15" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>11</v>
       </c>
@@ -4808,7 +4808,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="15" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>12</v>
       </c>
@@ -4848,7 +4848,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="75" customHeight="1" s="54">
       <c r="A15" t="inlineStr">
         <is>
           <t>Note: Participant IDs (P1–P12) are pseudonymised. * Investment Type and Sector apply to Tenant Representatives only. Signed consent forms are held by the researcher and available on request.</t>
@@ -5876,7 +5876,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" s="54">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>#</t>
@@ -5943,7 +5943,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" s="54">
+    <row r="3" ht="30" customHeight="1" s="54">
       <c r="A3" s="84" t="n"/>
       <c r="B3" s="84" t="n"/>
       <c r="C3" s="84" t="n"/>
@@ -5998,7 +5998,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1" s="54">
+    <row r="4" ht="45" customHeight="1" s="54">
       <c r="A4" s="85" t="inlineStr">
         <is>
           <t>Scale:  1 = Strongly Disagree    2 = Disagree    3 = Neutral    4 = Agree    5 = Strongly Agree</t>
@@ -6021,7 +6021,7 @@
       <c r="L4" s="28" t="n"/>
       <c r="M4" s="28" t="n"/>
     </row>
-    <row r="5" ht="19.5" customHeight="1" s="54">
+    <row r="5" ht="15" customHeight="1" s="54">
       <c r="A5" s="23" t="n">
         <v>1</v>
       </c>
@@ -6066,7 +6066,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" ht="19.5" customHeight="1" s="54">
+    <row r="6" ht="15" customHeight="1" s="54">
       <c r="A6" s="24" t="n">
         <v>2</v>
       </c>
@@ -6111,7 +6111,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" ht="19.5" customHeight="1" s="54">
+    <row r="7" ht="15" customHeight="1" s="54">
       <c r="A7" s="23" t="n">
         <v>3</v>
       </c>
@@ -6156,7 +6156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" ht="19.5" customHeight="1" s="54">
+    <row r="8" ht="15" customHeight="1" s="54">
       <c r="A8" s="24" t="n">
         <v>4</v>
       </c>
@@ -6201,7 +6201,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="19.5" customHeight="1" s="54">
+    <row r="9" ht="15" customHeight="1" s="54">
       <c r="A9" s="23" t="n">
         <v>5</v>
       </c>
@@ -6246,7 +6246,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" ht="19.5" customHeight="1" s="54">
+    <row r="10" ht="15" customHeight="1" s="54">
       <c r="A10" s="24" t="n">
         <v>6</v>
       </c>
@@ -6291,7 +6291,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" ht="19.5" customHeight="1" s="54">
+    <row r="11" ht="15" customHeight="1" s="54">
       <c r="A11" s="23" t="n">
         <v>7</v>
       </c>
@@ -6336,7 +6336,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" ht="19.5" customHeight="1" s="54">
+    <row r="12" ht="15" customHeight="1" s="54">
       <c r="A12" s="24" t="n">
         <v>8</v>
       </c>
@@ -6381,7 +6381,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" ht="19.5" customHeight="1" s="54">
+    <row r="13" ht="15" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>9</v>
       </c>
@@ -6426,7 +6426,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="15" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>10</v>
       </c>
@@ -6471,7 +6471,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" s="54">
+    <row r="15" ht="15" customHeight="1" s="54">
       <c r="A15" s="23" t="n">
         <v>11</v>
       </c>
@@ -6516,7 +6516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="15" customHeight="1" s="54">
       <c r="A16" s="23" t="n">
         <v>12</v>
       </c>
@@ -6561,7 +6561,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="45" customHeight="1" s="54">
       <c r="A17" t="inlineStr">
         <is>
           <t>⚠  Fill in each cell with the participant's actual response (integer 1–5). Scores in 'SUS Score Calculation' update automatically.</t>
@@ -7595,7 +7595,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" s="54">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>#</t>
@@ -7672,7 +7672,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" s="54">
+    <row r="3" ht="15" customHeight="1" s="54">
       <c r="A3" s="84" t="n"/>
       <c r="B3" s="84" t="n"/>
       <c r="C3" s="84" t="n"/>
@@ -7737,7 +7737,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="19.5" customHeight="1" s="54">
+    <row r="4" ht="30" customHeight="1" s="54">
       <c r="A4" s="23" t="n">
         <v>1</v>
       </c>
@@ -7800,7 +7800,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="19.5" customHeight="1" s="54">
+    <row r="5" ht="30" customHeight="1" s="54">
       <c r="A5" s="24" t="n">
         <v>2</v>
       </c>
@@ -7863,7 +7863,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="19.5" customHeight="1" s="54">
+    <row r="6" ht="30" customHeight="1" s="54">
       <c r="A6" s="23" t="n">
         <v>3</v>
       </c>
@@ -7926,7 +7926,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="19.5" customHeight="1" s="54">
+    <row r="7" ht="30" customHeight="1" s="54">
       <c r="A7" s="24" t="n">
         <v>4</v>
       </c>
@@ -7989,7 +7989,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="19.5" customHeight="1" s="54">
+    <row r="8" ht="30" customHeight="1" s="54">
       <c r="A8" s="23" t="n">
         <v>5</v>
       </c>
@@ -8052,7 +8052,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="19.5" customHeight="1" s="54">
+    <row r="9" ht="30" customHeight="1" s="54">
       <c r="A9" s="24" t="n">
         <v>6</v>
       </c>
@@ -8115,7 +8115,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="19.5" customHeight="1" s="54">
+    <row r="10" ht="45" customHeight="1" s="54">
       <c r="A10" s="23" t="n">
         <v>7</v>
       </c>
@@ -8178,7 +8178,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="19.5" customHeight="1" s="54">
+    <row r="11" ht="45" customHeight="1" s="54">
       <c r="A11" s="24" t="n">
         <v>8</v>
       </c>
@@ -8241,7 +8241,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="19.5" customHeight="1" s="54">
+    <row r="12" ht="45" customHeight="1" s="54">
       <c r="A12" s="23" t="n">
         <v>9</v>
       </c>
@@ -8304,7 +8304,7 @@
         <v/>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="45" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>10</v>
       </c>
@@ -8367,7 +8367,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1" s="54">
+    <row r="14" ht="45" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>11</v>
       </c>
@@ -8431,7 +8431,7 @@
       </c>
       <c r="P14" s="90" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="45" customHeight="1" s="54">
       <c r="A15" s="23" t="n">
         <v>12</v>
       </c>
@@ -8496,7 +8496,7 @@
       <c r="P15" s="90" t="n"/>
       <c r="Q15" s="90" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="15" customHeight="1" s="54">
       <c r="A16" s="91" t="inlineStr">
         <is>
           <t>MEAN SUS SCORE</t>
@@ -9534,14 +9534,14 @@
     <col width="8.7265625" customWidth="1" style="54" min="8" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" s="54">
+    <row r="1" ht="30" customHeight="1" s="54">
       <c r="A1" s="81" t="inlineStr">
         <is>
           <t>SUS Evaluation — Summary of Results | IPDC-OSS Platform</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" s="54">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>#</t>
@@ -9578,7 +9578,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="19.5" customHeight="1" s="54">
+    <row r="3" ht="45" customHeight="1" s="54">
       <c r="A3" s="23" t="n">
         <v>1</v>
       </c>
@@ -9610,7 +9610,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="19.5" customHeight="1" s="54">
+    <row r="4" ht="45" customHeight="1" s="54">
       <c r="A4" s="24" t="n">
         <v>2</v>
       </c>
@@ -9642,7 +9642,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="19.5" customHeight="1" s="54">
+    <row r="5" ht="45" customHeight="1" s="54">
       <c r="A5" s="23" t="n">
         <v>3</v>
       </c>
@@ -9674,7 +9674,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="19.5" customHeight="1" s="54">
+    <row r="6" ht="45" customHeight="1" s="54">
       <c r="A6" s="24" t="n">
         <v>4</v>
       </c>
@@ -9706,7 +9706,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="19.5" customHeight="1" s="54">
+    <row r="7" ht="45" customHeight="1" s="54">
       <c r="A7" s="23" t="n">
         <v>5</v>
       </c>
@@ -9738,7 +9738,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="19.5" customHeight="1" s="54">
+    <row r="8" ht="45" customHeight="1" s="54">
       <c r="A8" s="24" t="n">
         <v>6</v>
       </c>
@@ -9770,7 +9770,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="19.5" customHeight="1" s="54">
+    <row r="9" ht="45" customHeight="1" s="54">
       <c r="A9" s="23" t="n">
         <v>7</v>
       </c>
@@ -9802,7 +9802,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="19.5" customHeight="1" s="54">
+    <row r="10" ht="45" customHeight="1" s="54">
       <c r="A10" s="24" t="n">
         <v>8</v>
       </c>
@@ -9834,7 +9834,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="19.5" customHeight="1" s="54">
+    <row r="11" ht="45" customHeight="1" s="54">
       <c r="A11" s="23" t="n">
         <v>9</v>
       </c>
@@ -9866,7 +9866,7 @@
         <v/>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="45" customHeight="1" s="54">
       <c r="A12" s="23" t="n">
         <v>10</v>
       </c>
@@ -9898,7 +9898,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="25.5" customHeight="1" s="54">
+    <row r="13" ht="45" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>11</v>
       </c>
@@ -9931,7 +9931,7 @@
       </c>
       <c r="H13" s="90" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="45" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>12</v>
       </c>
@@ -9965,7 +9965,7 @@
       <c r="H14" s="90" t="n"/>
       <c r="I14" s="90" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="45" customHeight="1" s="54">
       <c r="A15" s="91" t="inlineStr">
         <is>
           <t>MEAN SUS SCORE</t>
@@ -9990,7 +9990,7 @@
       <c r="I15" s="90" t="n"/>
       <c r="J15" s="90" t="n"/>
     </row>
-    <row r="16" ht="15.75" customHeight="1" s="54">
+    <row r="16" ht="30" customHeight="1" s="54">
       <c r="A16" s="86" t="inlineStr">
         <is>
           <t>Reference lines: 72.5 = Good threshold | 85.5 = Excellent threshold</t>
@@ -11016,21 +11016,21 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" s="54">
+    <row r="2" ht="45" customHeight="1" s="54">
       <c r="A2" s="87" t="inlineStr">
         <is>
           <t>These questions are supplementary to the SUS — they do NOT affect the SUS score calculation.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" s="54">
+    <row r="3" ht="30" customHeight="1" s="54">
       <c r="A3" s="88" t="inlineStr">
         <is>
           <t>Q8b — Offline Tasks Attempted (tick = attempted)  |  Google Form: Section 6 of 9</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="49.5" customHeight="1" s="54">
+    <row r="4" ht="15" customHeight="1" s="54">
       <c r="A4" s="32" t="inlineStr">
         <is>
           <t>#</t>
@@ -11077,7 +11077,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1" s="54">
+    <row r="5" ht="15" customHeight="1" s="54">
       <c r="A5" s="23" t="n">
         <v>1</v>
       </c>
@@ -11114,7 +11114,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" s="54">
+    <row r="6" ht="15" customHeight="1" s="54">
       <c r="A6" s="24" t="n">
         <v>2</v>
       </c>
@@ -11139,7 +11139,7 @@
       <c r="H6" s="46" t="n"/>
       <c r="I6" s="46" t="n"/>
     </row>
-    <row r="7" ht="18" customHeight="1" s="54">
+    <row r="7" ht="15" customHeight="1" s="54">
       <c r="A7" s="23" t="n">
         <v>3</v>
       </c>
@@ -11164,7 +11164,7 @@
       <c r="H7" s="46" t="n"/>
       <c r="I7" s="46" t="n"/>
     </row>
-    <row r="8" ht="18" customHeight="1" s="54">
+    <row r="8" ht="15" customHeight="1" s="54">
       <c r="A8" s="24" t="n">
         <v>4</v>
       </c>
@@ -11189,7 +11189,7 @@
       <c r="H8" s="46" t="n"/>
       <c r="I8" s="46" t="n"/>
     </row>
-    <row r="9" ht="18" customHeight="1" s="54">
+    <row r="9" ht="15" customHeight="1" s="54">
       <c r="A9" s="23" t="n">
         <v>5</v>
       </c>
@@ -11214,7 +11214,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="54">
+    <row r="10" ht="15" customHeight="1" s="54">
       <c r="A10" s="24" t="n">
         <v>6</v>
       </c>
@@ -11239,7 +11239,7 @@
       <c r="H10" s="46" t="n"/>
       <c r="I10" s="46" t="n"/>
     </row>
-    <row r="11" ht="18" customHeight="1" s="54">
+    <row r="11" ht="15" customHeight="1" s="54">
       <c r="A11" s="23" t="n">
         <v>7</v>
       </c>
@@ -11280,7 +11280,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" s="54">
+    <row r="12" ht="15" customHeight="1" s="54">
       <c r="A12" s="24" t="n">
         <v>8</v>
       </c>
@@ -11309,7 +11309,7 @@
       <c r="H12" s="46" t="n"/>
       <c r="I12" s="46" t="n"/>
     </row>
-    <row r="13" ht="18" customHeight="1" s="54">
+    <row r="13" ht="15" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>9</v>
       </c>
@@ -11354,7 +11354,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="15" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>10</v>
       </c>
@@ -11379,7 +11379,7 @@
       <c r="H14" s="46" t="n"/>
       <c r="I14" s="46" t="n"/>
     </row>
-    <row r="15" ht="14.5" customHeight="1" s="54">
+    <row r="15" ht="15" customHeight="1" s="54">
       <c r="A15" s="23" t="n">
         <v>11</v>
       </c>
@@ -11404,7 +11404,7 @@
       <c r="H15" s="46" t="n"/>
       <c r="I15" s="46" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="15" customHeight="1" s="54">
       <c r="A16" s="23" t="n">
         <v>12</v>
       </c>
@@ -11441,7 +11441,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" s="54">
+    <row r="17" ht="30" customHeight="1" s="54">
       <c r="A17" s="87" t="inlineStr">
         <is>
           <t>Enter  ✓  if the participant attempted the task, or leave blank if not attempted.</t>
@@ -11457,7 +11457,7 @@
       <c r="I17" s="90" t="n"/>
       <c r="J17" s="90" t="n"/>
     </row>
-    <row r="18" ht="43.5" customHeight="1" s="54">
+    <row r="18" ht="15" customHeight="1" s="54">
       <c r="A18" s="92" t="n"/>
       <c r="B18" s="92" t="n"/>
       <c r="C18" s="92" t="n"/>
@@ -11468,7 +11468,7 @@
       <c r="H18" s="92" t="n"/>
       <c r="I18" s="92" t="n"/>
     </row>
-    <row r="19" ht="18" customHeight="1" s="54">
+    <row r="19" ht="45" customHeight="1" s="54">
       <c r="A19" s="88" t="inlineStr">
         <is>
           <t>Q19 — Offline Confidence Score  |  Q20 — Online/Offline Clarity  |  Google Form: Section 8 of 9</t>
@@ -11485,7 +11485,7 @@
       <c r="J19" s="90" t="n"/>
       <c r="K19" s="90" t="n"/>
     </row>
-    <row r="20" ht="18" customHeight="1" s="54">
+    <row r="20" ht="30" customHeight="1" s="54">
       <c r="A20" s="32" t="inlineStr">
         <is>
           <t>#</t>
@@ -11521,7 +11521,7 @@
       <c r="K20" s="90" t="n"/>
       <c r="L20" s="90" t="n"/>
     </row>
-    <row r="21" ht="18" customHeight="1" s="54">
+    <row r="21" ht="15" customHeight="1" s="54">
       <c r="A21" s="23" t="n">
         <v>1</v>
       </c>
@@ -11544,7 +11544,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1" s="54">
+    <row r="22" ht="15" customHeight="1" s="54">
       <c r="A22" s="24" t="n">
         <v>2</v>
       </c>
@@ -11567,7 +11567,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1" s="54">
+    <row r="23" ht="15" customHeight="1" s="54">
       <c r="A23" s="23" t="n">
         <v>3</v>
       </c>
@@ -11590,7 +11590,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1" s="54">
+    <row r="24" ht="15" customHeight="1" s="54">
       <c r="A24" s="24" t="n">
         <v>4</v>
       </c>
@@ -11613,7 +11613,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1" s="54">
+    <row r="25" ht="15" customHeight="1" s="54">
       <c r="A25" s="23" t="n">
         <v>5</v>
       </c>
@@ -11636,7 +11636,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1" s="54">
+    <row r="26" ht="15" customHeight="1" s="54">
       <c r="A26" s="24" t="n">
         <v>6</v>
       </c>
@@ -11659,7 +11659,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1" s="54">
+    <row r="27" ht="15" customHeight="1" s="54">
       <c r="A27" s="23" t="n">
         <v>7</v>
       </c>
@@ -11682,7 +11682,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="21.75" customHeight="1" s="54">
+    <row r="28" ht="15" customHeight="1" s="54">
       <c r="A28" s="23" t="n">
         <v>8</v>
       </c>
@@ -11713,7 +11713,7 @@
       <c r="L28" s="90" t="n"/>
       <c r="M28" s="90" t="n"/>
     </row>
-    <row r="29" ht="15.75" customHeight="1" s="54">
+    <row r="29" ht="15" customHeight="1" s="54">
       <c r="A29" s="23" t="n">
         <v>9</v>
       </c>
@@ -11745,7 +11745,7 @@
       <c r="M29" s="90" t="n"/>
       <c r="N29" s="90" t="n"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="54">
+    <row r="30" ht="15" customHeight="1" s="54">
       <c r="A30" s="23" t="n">
         <v>10</v>
       </c>
@@ -11778,7 +11778,7 @@
       <c r="N30" s="90" t="n"/>
       <c r="O30" s="90" t="n"/>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="54">
+    <row r="31" ht="15" customHeight="1" s="54">
       <c r="A31" s="23" t="n">
         <v>11</v>
       </c>
@@ -11812,7 +11812,7 @@
       <c r="O31" s="90" t="n"/>
       <c r="P31" s="90" t="n"/>
     </row>
-    <row r="32" ht="15.75" customHeight="1" s="54">
+    <row r="32" ht="15" customHeight="1" s="54">
       <c r="A32" s="23" t="n">
         <v>12</v>
       </c>
@@ -11847,7 +11847,7 @@
       <c r="P32" s="90" t="n"/>
       <c r="Q32" s="90" t="n"/>
     </row>
-    <row r="33" ht="15.75" customHeight="1" s="54">
+    <row r="33" ht="15" customHeight="1" s="54">
       <c r="A33" s="91" t="inlineStr">
         <is>
           <t>MEAN (Q19)</t>

</xml_diff>

<commit_message>
Fix: Improve row height calculation with wrap-aware line estimation
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/research/SUS_Evaluation_IPDC_OSS.xlsx
+++ b/data/research/SUS_Evaluation_IPDC_OSS.xlsx
@@ -1430,7 +1430,7 @@
     <col width="21.54296875" customWidth="1" style="54" min="29" max="34"/>
   </cols>
   <sheetData>
-    <row r="1" ht="60" customHeight="1" s="54">
+    <row r="1" ht="45" customHeight="1" s="54">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Timestamp</t>
@@ -1582,7 +1582,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1" s="54">
+    <row r="2" ht="75" customHeight="1" s="54">
       <c r="A2" s="5" t="n">
         <v>46090.50363871528</v>
       </c>
@@ -1680,7 +1680,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" s="54">
+    <row r="3" ht="18" customHeight="1" s="54">
       <c r="A3" s="5" t="n">
         <v>46097.05842277778</v>
       </c>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="AB3" s="48" t="n"/>
     </row>
-    <row r="4" ht="30" customHeight="1" s="54">
+    <row r="4" ht="18" customHeight="1" s="54">
       <c r="A4" s="5" t="n">
         <v>46099.23142234953</v>
       </c>
@@ -2063,7 +2063,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" s="54">
+    <row r="7" ht="45" customHeight="1" s="54">
       <c r="A7" s="5" t="n">
         <v>46099.25578788194</v>
       </c>
@@ -2156,7 +2156,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="105" customHeight="1" s="54">
+    <row r="8" ht="90" customHeight="1" s="54">
       <c r="A8" s="5" t="n">
         <v>46099.25783776621</v>
       </c>
@@ -2249,7 +2249,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" s="54">
+    <row r="9" ht="45" customHeight="1" s="54">
       <c r="A9" s="5" t="n">
         <v>46099.26724091435</v>
       </c>
@@ -2342,7 +2342,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="120" customHeight="1" s="54">
+    <row r="10" ht="105" customHeight="1" s="54">
       <c r="A10" s="5" t="n">
         <v>46099.2790071875</v>
       </c>
@@ -2627,7 +2627,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="90" customHeight="1" s="54">
+    <row r="13" ht="75" customHeight="1" s="54">
       <c r="A13" s="5" t="n">
         <v>46103.97938486111</v>
       </c>
@@ -2773,23 +2773,23 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="54"/>
-    <row r="4" ht="15" customHeight="1" s="54">
+    <row r="3" ht="18" customHeight="1" s="54"/>
+    <row r="4" ht="18" customHeight="1" s="54">
       <c r="A4" s="74" t="inlineStr">
         <is>
           <t>PURPOSE</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="105" customHeight="1" s="54">
+    <row r="5" ht="90" customHeight="1" s="54">
       <c r="A5" s="75" t="inlineStr">
         <is>
           <t>This workbook is the official data collection and calculation instrument for the SUS usability evaluation of the IPDC Digital One-Stop-Service (OSS) platform prototype. It accompanies the thesis: 'Design and Development of a Digital One-Stop-Service Platform for Industrial Parks in Ethiopia'.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="54"/>
-    <row r="7" ht="15" customHeight="1" s="54">
+    <row r="6" ht="18" customHeight="1" s="54"/>
+    <row r="7" ht="18" customHeight="1" s="54">
       <c r="A7" s="74" t="inlineStr">
         <is>
           <t>WORKBOOK STRUCTURE</t>
@@ -2874,15 +2874,15 @@
       </c>
       <c r="D13" s="77" t="n"/>
     </row>
-    <row r="14" ht="15" customHeight="1" s="54"/>
-    <row r="15" ht="15" customHeight="1" s="54">
+    <row r="14" ht="18" customHeight="1" s="54"/>
+    <row r="15" ht="18" customHeight="1" s="54">
       <c r="A15" s="74" t="inlineStr">
         <is>
           <t>SUS SCORING FORMULA</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="54">
+    <row r="16" ht="18" customHeight="1" s="54">
       <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Odd items — Positive (Q1,Q3,Q5,Q7,Q9):</t>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="D16" s="77" t="n"/>
     </row>
-    <row r="17" ht="15" customHeight="1" s="54">
+    <row r="17" ht="18" customHeight="1" s="54">
       <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Even items — Negative (Q2,Q4,Q6,Q8,Q10):</t>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="D17" s="77" t="n"/>
     </row>
-    <row r="18" ht="15" customHeight="1" s="54">
+    <row r="18" ht="18" customHeight="1" s="54">
       <c r="B18" s="8" t="inlineStr">
         <is>
           <t>SUS Score:</t>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="D18" s="77" t="n"/>
     </row>
-    <row r="19" ht="15" customHeight="1" s="54">
+    <row r="19" ht="18" customHeight="1" s="54">
       <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Scale:</t>
@@ -2934,15 +2934,15 @@
       </c>
       <c r="D19" s="77" t="n"/>
     </row>
-    <row r="20" ht="15" customHeight="1" s="54"/>
-    <row r="21" ht="30" customHeight="1" s="54">
+    <row r="20" ht="18" customHeight="1" s="54"/>
+    <row r="21" ht="18" customHeight="1" s="54">
       <c r="A21" s="74" t="inlineStr">
         <is>
           <t>SUS SCORE INTERPRETATION (Bangor et al. / Sauro)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="54">
+    <row r="22" ht="18" customHeight="1" s="54">
       <c r="B22" s="9" t="inlineStr">
         <is>
           <t>&gt; 85.5</t>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="54">
+    <row r="23" ht="18" customHeight="1" s="54">
       <c r="B23" s="11" t="inlineStr">
         <is>
           <t>72.6 – 85.5</t>
@@ -2976,7 +2976,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="54">
+    <row r="24" ht="18" customHeight="1" s="54">
       <c r="B24" s="13" t="inlineStr">
         <is>
           <t>52.0 – 72.5</t>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="54">
+    <row r="25" ht="18" customHeight="1" s="54">
       <c r="B25" s="15" t="inlineStr">
         <is>
           <t>51.7 – 51.9</t>
@@ -3010,7 +3010,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="54">
+    <row r="26" ht="18" customHeight="1" s="54">
       <c r="B26" s="17" t="inlineStr">
         <is>
           <t>&lt; 51.6</t>
@@ -3027,8 +3027,8 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="54"/>
-    <row r="28" ht="15" customHeight="1" s="54">
+    <row r="27" ht="18" customHeight="1" s="54"/>
+    <row r="28" ht="18" customHeight="1" s="54">
       <c r="A28" s="74" t="inlineStr">
         <is>
           <t>TASK SCENARIOS ADMINISTERED TO PARTICIPANTS</t>
@@ -3069,7 +3069,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="45" customHeight="1" s="54">
+    <row r="31" ht="30" customHeight="1" s="54">
       <c r="B31" s="19" t="inlineStr">
         <is>
           <t>Task M3</t>
@@ -3086,7 +3086,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="45" customHeight="1" s="54">
+    <row r="32" ht="30" customHeight="1" s="54">
       <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Task M4</t>
@@ -3120,7 +3120,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="45" customHeight="1" s="54">
+    <row r="34" ht="30" customHeight="1" s="54">
       <c r="B34" s="19" t="inlineStr">
         <is>
           <t>Task T2</t>
@@ -3154,7 +3154,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="45" customHeight="1" s="54">
+    <row r="36" ht="30" customHeight="1" s="54">
       <c r="B36" s="19" t="inlineStr">
         <is>
           <t>Task T4</t>
@@ -3171,7 +3171,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="45" customHeight="1" s="54">
+    <row r="37" ht="30" customHeight="1" s="54">
       <c r="B37" s="19" t="inlineStr">
         <is>
           <t>Task O1</t>
@@ -3188,7 +3188,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="45" customHeight="1" s="54">
+    <row r="38" ht="30" customHeight="1" s="54">
       <c r="B38" s="19" t="inlineStr">
         <is>
           <t>Task O2</t>
@@ -3222,7 +3222,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="45" customHeight="1" s="54">
+    <row r="40" ht="30" customHeight="1" s="54">
       <c r="B40" s="19" t="inlineStr">
         <is>
           <t>Task O4</t>
@@ -3239,7 +3239,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="45" customHeight="1" s="54">
+    <row r="41" ht="30" customHeight="1" s="54">
       <c r="B41" s="19" t="inlineStr">
         <is>
           <t>Task X1</t>
@@ -3256,7 +3256,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="45" customHeight="1" s="54">
+    <row r="42" ht="30" customHeight="1" s="54">
       <c r="B42" s="19" t="inlineStr">
         <is>
           <t>Task X2</t>
@@ -3290,7 +3290,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="45" customHeight="1" s="54">
+    <row r="44" ht="30" customHeight="1" s="54">
       <c r="B44" s="19" t="inlineStr">
         <is>
           <t>Task X4</t>
@@ -3307,8 +3307,8 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1" s="54"/>
-    <row r="46" ht="90" customHeight="1" s="54">
+    <row r="45" ht="18" customHeight="1" s="54"/>
+    <row r="46" ht="75" customHeight="1" s="54">
       <c r="A46" s="79" t="inlineStr">
         <is>
           <t>⚠  IMPORTANT: Enter REAL participant responses in the 'SUS Raw Responses' sheet. All SUS scores in the thesis must reflect actual collected data. Scores in 'SUS Score Calculation' and 'Summary &amp; Results' update automatically.</t>
@@ -4319,14 +4319,14 @@
     <col width="8.7265625" customWidth="1" style="54" min="9" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1" s="54">
+    <row r="1" ht="30" customHeight="1" s="54">
       <c r="A1" s="81" t="inlineStr">
         <is>
           <t>Usability Evaluation — Participant Profiles (9–18 March 2026 | 12 Participants | Chapter 5)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="54">
+    <row r="2" ht="18" customHeight="1" s="54">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>#</t>
@@ -4368,7 +4368,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="54">
+    <row r="3" ht="18" customHeight="1" s="54">
       <c r="A3" s="23" t="n">
         <v>1</v>
       </c>
@@ -4408,7 +4408,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="54">
+    <row r="4" ht="18" customHeight="1" s="54">
       <c r="A4" s="24" t="n">
         <v>2</v>
       </c>
@@ -4448,7 +4448,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="54">
+    <row r="5" ht="18" customHeight="1" s="54">
       <c r="A5" s="23" t="n">
         <v>3</v>
       </c>
@@ -4488,7 +4488,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="54">
+    <row r="6" ht="18" customHeight="1" s="54">
       <c r="A6" s="24" t="n">
         <v>4</v>
       </c>
@@ -4528,7 +4528,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="54">
+    <row r="7" ht="18" customHeight="1" s="54">
       <c r="A7" s="23" t="n">
         <v>5</v>
       </c>
@@ -4568,7 +4568,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="54">
+    <row r="8" ht="18" customHeight="1" s="54">
       <c r="A8" s="24" t="n">
         <v>6</v>
       </c>
@@ -4608,7 +4608,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="54">
+    <row r="9" ht="18" customHeight="1" s="54">
       <c r="A9" s="23" t="n">
         <v>7</v>
       </c>
@@ -4648,7 +4648,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="54">
+    <row r="10" ht="18" customHeight="1" s="54">
       <c r="A10" s="24" t="n">
         <v>8</v>
       </c>
@@ -4688,7 +4688,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="54">
+    <row r="11" ht="18" customHeight="1" s="54">
       <c r="A11" s="23" t="n">
         <v>9</v>
       </c>
@@ -4728,7 +4728,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="54">
+    <row r="12" ht="18" customHeight="1" s="54">
       <c r="A12" s="23" t="n">
         <v>10</v>
       </c>
@@ -4768,7 +4768,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="54">
+    <row r="13" ht="18" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>11</v>
       </c>
@@ -4808,7 +4808,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="54">
+    <row r="14" ht="18" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>12</v>
       </c>
@@ -4848,7 +4848,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="75" customHeight="1" s="54">
+    <row r="15" ht="60" customHeight="1" s="54">
       <c r="A15" t="inlineStr">
         <is>
           <t>Note: Participant IDs (P1–P12) are pseudonymised. * Investment Type and Sector apply to Tenant Representatives only. Signed consent forms are held by the researcher and available on request.</t>
@@ -5876,7 +5876,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="54">
+    <row r="2" ht="18" customHeight="1" s="54">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>#</t>
@@ -5998,7 +5998,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1" s="54">
+    <row r="4" ht="30" customHeight="1" s="54">
       <c r="A4" s="85" t="inlineStr">
         <is>
           <t>Scale:  1 = Strongly Disagree    2 = Disagree    3 = Neutral    4 = Agree    5 = Strongly Agree</t>
@@ -6021,7 +6021,7 @@
       <c r="L4" s="28" t="n"/>
       <c r="M4" s="28" t="n"/>
     </row>
-    <row r="5" ht="15" customHeight="1" s="54">
+    <row r="5" ht="18" customHeight="1" s="54">
       <c r="A5" s="23" t="n">
         <v>1</v>
       </c>
@@ -6066,7 +6066,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="54">
+    <row r="6" ht="18" customHeight="1" s="54">
       <c r="A6" s="24" t="n">
         <v>2</v>
       </c>
@@ -6111,7 +6111,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="54">
+    <row r="7" ht="18" customHeight="1" s="54">
       <c r="A7" s="23" t="n">
         <v>3</v>
       </c>
@@ -6156,7 +6156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="54">
+    <row r="8" ht="18" customHeight="1" s="54">
       <c r="A8" s="24" t="n">
         <v>4</v>
       </c>
@@ -6201,7 +6201,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="54">
+    <row r="9" ht="18" customHeight="1" s="54">
       <c r="A9" s="23" t="n">
         <v>5</v>
       </c>
@@ -6246,7 +6246,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="54">
+    <row r="10" ht="18" customHeight="1" s="54">
       <c r="A10" s="24" t="n">
         <v>6</v>
       </c>
@@ -6291,7 +6291,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="54">
+    <row r="11" ht="18" customHeight="1" s="54">
       <c r="A11" s="23" t="n">
         <v>7</v>
       </c>
@@ -6336,7 +6336,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="54">
+    <row r="12" ht="18" customHeight="1" s="54">
       <c r="A12" s="24" t="n">
         <v>8</v>
       </c>
@@ -6381,7 +6381,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="54">
+    <row r="13" ht="18" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>9</v>
       </c>
@@ -6426,7 +6426,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="54">
+    <row r="14" ht="18" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>10</v>
       </c>
@@ -6471,7 +6471,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="54">
+    <row r="15" ht="18" customHeight="1" s="54">
       <c r="A15" s="23" t="n">
         <v>11</v>
       </c>
@@ -6516,7 +6516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="54">
+    <row r="16" ht="18" customHeight="1" s="54">
       <c r="A16" s="23" t="n">
         <v>12</v>
       </c>
@@ -7595,7 +7595,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="54">
+    <row r="2" ht="18" customHeight="1" s="54">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>#</t>
@@ -7672,7 +7672,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="54">
+    <row r="3" ht="18" customHeight="1" s="54">
       <c r="A3" s="84" t="n"/>
       <c r="B3" s="84" t="n"/>
       <c r="C3" s="84" t="n"/>
@@ -8115,7 +8115,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="45" customHeight="1" s="54">
+    <row r="10" ht="30" customHeight="1" s="54">
       <c r="A10" s="23" t="n">
         <v>7</v>
       </c>
@@ -8178,7 +8178,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1" s="54">
+    <row r="11" ht="30" customHeight="1" s="54">
       <c r="A11" s="24" t="n">
         <v>8</v>
       </c>
@@ -8241,7 +8241,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="45" customHeight="1" s="54">
+    <row r="12" ht="30" customHeight="1" s="54">
       <c r="A12" s="23" t="n">
         <v>9</v>
       </c>
@@ -8304,7 +8304,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1" s="54">
+    <row r="13" ht="30" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>10</v>
       </c>
@@ -8367,7 +8367,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1" s="54">
+    <row r="14" ht="30" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>11</v>
       </c>
@@ -8431,7 +8431,7 @@
       </c>
       <c r="P14" s="90" t="n"/>
     </row>
-    <row r="15" ht="45" customHeight="1" s="54">
+    <row r="15" ht="30" customHeight="1" s="54">
       <c r="A15" s="23" t="n">
         <v>12</v>
       </c>
@@ -8496,7 +8496,7 @@
       <c r="P15" s="90" t="n"/>
       <c r="Q15" s="90" t="n"/>
     </row>
-    <row r="16" ht="15" customHeight="1" s="54">
+    <row r="16" ht="18" customHeight="1" s="54">
       <c r="A16" s="91" t="inlineStr">
         <is>
           <t>MEAN SUS SCORE</t>
@@ -9541,7 +9541,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="54">
+    <row r="2" ht="18" customHeight="1" s="54">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>#</t>
@@ -9578,7 +9578,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1" s="54">
+    <row r="3" ht="30" customHeight="1" s="54">
       <c r="A3" s="23" t="n">
         <v>1</v>
       </c>
@@ -9610,7 +9610,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1" s="54">
+    <row r="4" ht="30" customHeight="1" s="54">
       <c r="A4" s="24" t="n">
         <v>2</v>
       </c>
@@ -9642,7 +9642,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1" s="54">
+    <row r="5" ht="30" customHeight="1" s="54">
       <c r="A5" s="23" t="n">
         <v>3</v>
       </c>
@@ -9674,7 +9674,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1" s="54">
+    <row r="6" ht="30" customHeight="1" s="54">
       <c r="A6" s="24" t="n">
         <v>4</v>
       </c>
@@ -9706,7 +9706,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1" s="54">
+    <row r="7" ht="30" customHeight="1" s="54">
       <c r="A7" s="23" t="n">
         <v>5</v>
       </c>
@@ -9738,7 +9738,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1" s="54">
+    <row r="8" ht="30" customHeight="1" s="54">
       <c r="A8" s="24" t="n">
         <v>6</v>
       </c>
@@ -9770,7 +9770,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1" s="54">
+    <row r="9" ht="30" customHeight="1" s="54">
       <c r="A9" s="23" t="n">
         <v>7</v>
       </c>
@@ -9802,7 +9802,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="45" customHeight="1" s="54">
+    <row r="10" ht="30" customHeight="1" s="54">
       <c r="A10" s="24" t="n">
         <v>8</v>
       </c>
@@ -9834,7 +9834,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1" s="54">
+    <row r="11" ht="30" customHeight="1" s="54">
       <c r="A11" s="23" t="n">
         <v>9</v>
       </c>
@@ -9866,7 +9866,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="45" customHeight="1" s="54">
+    <row r="12" ht="30" customHeight="1" s="54">
       <c r="A12" s="23" t="n">
         <v>10</v>
       </c>
@@ -9898,7 +9898,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1" s="54">
+    <row r="13" ht="30" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>11</v>
       </c>
@@ -9931,7 +9931,7 @@
       </c>
       <c r="H13" s="90" t="n"/>
     </row>
-    <row r="14" ht="45" customHeight="1" s="54">
+    <row r="14" ht="30" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>12</v>
       </c>
@@ -9965,7 +9965,7 @@
       <c r="H14" s="90" t="n"/>
       <c r="I14" s="90" t="n"/>
     </row>
-    <row r="15" ht="45" customHeight="1" s="54">
+    <row r="15" ht="30" customHeight="1" s="54">
       <c r="A15" s="91" t="inlineStr">
         <is>
           <t>MEAN SUS SCORE</t>
@@ -11016,7 +11016,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1" s="54">
+    <row r="2" ht="30" customHeight="1" s="54">
       <c r="A2" s="87" t="inlineStr">
         <is>
           <t>These questions are supplementary to the SUS — they do NOT affect the SUS score calculation.</t>
@@ -11030,7 +11030,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="54">
+    <row r="4" ht="18" customHeight="1" s="54">
       <c r="A4" s="32" t="inlineStr">
         <is>
           <t>#</t>
@@ -11077,7 +11077,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="54">
+    <row r="5" ht="18" customHeight="1" s="54">
       <c r="A5" s="23" t="n">
         <v>1</v>
       </c>
@@ -11114,7 +11114,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="54">
+    <row r="6" ht="18" customHeight="1" s="54">
       <c r="A6" s="24" t="n">
         <v>2</v>
       </c>
@@ -11139,7 +11139,7 @@
       <c r="H6" s="46" t="n"/>
       <c r="I6" s="46" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1" s="54">
+    <row r="7" ht="18" customHeight="1" s="54">
       <c r="A7" s="23" t="n">
         <v>3</v>
       </c>
@@ -11164,7 +11164,7 @@
       <c r="H7" s="46" t="n"/>
       <c r="I7" s="46" t="n"/>
     </row>
-    <row r="8" ht="15" customHeight="1" s="54">
+    <row r="8" ht="18" customHeight="1" s="54">
       <c r="A8" s="24" t="n">
         <v>4</v>
       </c>
@@ -11189,7 +11189,7 @@
       <c r="H8" s="46" t="n"/>
       <c r="I8" s="46" t="n"/>
     </row>
-    <row r="9" ht="15" customHeight="1" s="54">
+    <row r="9" ht="18" customHeight="1" s="54">
       <c r="A9" s="23" t="n">
         <v>5</v>
       </c>
@@ -11214,7 +11214,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="54">
+    <row r="10" ht="18" customHeight="1" s="54">
       <c r="A10" s="24" t="n">
         <v>6</v>
       </c>
@@ -11239,7 +11239,7 @@
       <c r="H10" s="46" t="n"/>
       <c r="I10" s="46" t="n"/>
     </row>
-    <row r="11" ht="15" customHeight="1" s="54">
+    <row r="11" ht="18" customHeight="1" s="54">
       <c r="A11" s="23" t="n">
         <v>7</v>
       </c>
@@ -11280,7 +11280,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="54">
+    <row r="12" ht="18" customHeight="1" s="54">
       <c r="A12" s="24" t="n">
         <v>8</v>
       </c>
@@ -11309,7 +11309,7 @@
       <c r="H12" s="46" t="n"/>
       <c r="I12" s="46" t="n"/>
     </row>
-    <row r="13" ht="15" customHeight="1" s="54">
+    <row r="13" ht="18" customHeight="1" s="54">
       <c r="A13" s="23" t="n">
         <v>9</v>
       </c>
@@ -11354,7 +11354,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="54">
+    <row r="14" ht="18" customHeight="1" s="54">
       <c r="A14" s="23" t="n">
         <v>10</v>
       </c>
@@ -11379,7 +11379,7 @@
       <c r="H14" s="46" t="n"/>
       <c r="I14" s="46" t="n"/>
     </row>
-    <row r="15" ht="15" customHeight="1" s="54">
+    <row r="15" ht="18" customHeight="1" s="54">
       <c r="A15" s="23" t="n">
         <v>11</v>
       </c>
@@ -11404,7 +11404,7 @@
       <c r="H15" s="46" t="n"/>
       <c r="I15" s="46" t="n"/>
     </row>
-    <row r="16" ht="15" customHeight="1" s="54">
+    <row r="16" ht="18" customHeight="1" s="54">
       <c r="A16" s="23" t="n">
         <v>12</v>
       </c>
@@ -11457,7 +11457,7 @@
       <c r="I17" s="90" t="n"/>
       <c r="J17" s="90" t="n"/>
     </row>
-    <row r="18" ht="15" customHeight="1" s="54">
+    <row r="18" ht="18" customHeight="1" s="54">
       <c r="A18" s="92" t="n"/>
       <c r="B18" s="92" t="n"/>
       <c r="C18" s="92" t="n"/>
@@ -11468,7 +11468,7 @@
       <c r="H18" s="92" t="n"/>
       <c r="I18" s="92" t="n"/>
     </row>
-    <row r="19" ht="45" customHeight="1" s="54">
+    <row r="19" ht="30" customHeight="1" s="54">
       <c r="A19" s="88" t="inlineStr">
         <is>
           <t>Q19 — Offline Confidence Score  |  Q20 — Online/Offline Clarity  |  Google Form: Section 8 of 9</t>
@@ -11521,7 +11521,7 @@
       <c r="K20" s="90" t="n"/>
       <c r="L20" s="90" t="n"/>
     </row>
-    <row r="21" ht="15" customHeight="1" s="54">
+    <row r="21" ht="18" customHeight="1" s="54">
       <c r="A21" s="23" t="n">
         <v>1</v>
       </c>
@@ -11544,7 +11544,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="54">
+    <row r="22" ht="18" customHeight="1" s="54">
       <c r="A22" s="24" t="n">
         <v>2</v>
       </c>
@@ -11567,7 +11567,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="54">
+    <row r="23" ht="18" customHeight="1" s="54">
       <c r="A23" s="23" t="n">
         <v>3</v>
       </c>
@@ -11590,7 +11590,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="54">
+    <row r="24" ht="18" customHeight="1" s="54">
       <c r="A24" s="24" t="n">
         <v>4</v>
       </c>
@@ -11613,7 +11613,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="54">
+    <row r="25" ht="18" customHeight="1" s="54">
       <c r="A25" s="23" t="n">
         <v>5</v>
       </c>
@@ -11636,7 +11636,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="54">
+    <row r="26" ht="18" customHeight="1" s="54">
       <c r="A26" s="24" t="n">
         <v>6</v>
       </c>
@@ -11659,7 +11659,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="54">
+    <row r="27" ht="18" customHeight="1" s="54">
       <c r="A27" s="23" t="n">
         <v>7</v>
       </c>
@@ -11682,7 +11682,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="54">
+    <row r="28" ht="18" customHeight="1" s="54">
       <c r="A28" s="23" t="n">
         <v>8</v>
       </c>
@@ -11713,7 +11713,7 @@
       <c r="L28" s="90" t="n"/>
       <c r="M28" s="90" t="n"/>
     </row>
-    <row r="29" ht="15" customHeight="1" s="54">
+    <row r="29" ht="18" customHeight="1" s="54">
       <c r="A29" s="23" t="n">
         <v>9</v>
       </c>
@@ -11745,7 +11745,7 @@
       <c r="M29" s="90" t="n"/>
       <c r="N29" s="90" t="n"/>
     </row>
-    <row r="30" ht="15" customHeight="1" s="54">
+    <row r="30" ht="18" customHeight="1" s="54">
       <c r="A30" s="23" t="n">
         <v>10</v>
       </c>
@@ -11778,7 +11778,7 @@
       <c r="N30" s="90" t="n"/>
       <c r="O30" s="90" t="n"/>
     </row>
-    <row r="31" ht="15" customHeight="1" s="54">
+    <row r="31" ht="18" customHeight="1" s="54">
       <c r="A31" s="23" t="n">
         <v>11</v>
       </c>
@@ -11812,7 +11812,7 @@
       <c r="O31" s="90" t="n"/>
       <c r="P31" s="90" t="n"/>
     </row>
-    <row r="32" ht="15" customHeight="1" s="54">
+    <row r="32" ht="18" customHeight="1" s="54">
       <c r="A32" s="23" t="n">
         <v>12</v>
       </c>
@@ -11847,7 +11847,7 @@
       <c r="P32" s="90" t="n"/>
       <c r="Q32" s="90" t="n"/>
     </row>
-    <row r="33" ht="15" customHeight="1" s="54">
+    <row r="33" ht="18" customHeight="1" s="54">
       <c r="A33" s="91" t="inlineStr">
         <is>
           <t>MEAN (Q19)</t>

</xml_diff>

<commit_message>
Fix: Update chart data range to include all 12 participants (P1-P12)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/research/SUS_Evaluation_IPDC_OSS.xlsx
+++ b/data/research/SUS_Evaluation_IPDC_OSS.xlsx
@@ -880,9 +880,9 @@
           <invertIfNegative val="1"/>
           <cat>
             <strRef>
-              <f>'Summary &amp; Results'!$B$3:$B$11</f>
+              <f>'Summary &amp; Results'!$B$3:$B$14</f>
               <strCache>
-                <ptCount val="9"/>
+                <ptCount val="12"/>
                 <pt idx="0">
                   <v>P1</v>
                 </pt>
@@ -910,42 +910,24 @@
                 <pt idx="8">
                   <v>P9</v>
                 </pt>
+                <pt idx="9">
+                  <v>P10</v>
+                </pt>
+                <pt idx="10">
+                  <v>P11</v>
+                </pt>
+                <pt idx="11">
+                  <v>P12</v>
+                </pt>
               </strCache>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary &amp; Results'!$E$3:$E$11</f>
+              <f>'Summary &amp; Results'!$E$3:$E$14</f>
               <numCache>
                 <formatCode>0.0</formatCode>
-                <ptCount val="9"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
+                <ptCount val="12"/>
               </numCache>
             </numRef>
           </val>

</xml_diff>